<commit_message>
docs: update test checklists for the dev's dashboard/AI features
Reflect the newly-integrated endpoints (PR #74) + the dashboard honesty cleanup
in both the markdown checklist and the regenerated QA workbook.

- 1.7: richer dashboard summary (greeting/KPIs "Coming Soon"/per-card error+Retry/
  real "Next 7 days"); 1.8: briefing "Do it" is backend-blocked (no action endpoint).
- New: 1.12 dashboard honest error+Retry, 1.13 activity feed (real actors + paging),
  1.14 onboarding AI panel, 5.9 AI budget guardrail (GET /ai/status).
- Backend-blocked list + "Known - not ready" tab: added the briefing action.
- Regenerated Cofoundaz_QA_Test_Sheet.xlsx from the generator (50 → 54 cases).
</commit_message>
<xml_diff>
--- a/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
+++ b/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
@@ -882,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1253,17 +1253,17 @@
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>The action is accepted and the page does not crash.</t>
+          <t>It acknowledges locally; the page doesn’t crash.</t>
         </is>
       </c>
       <c r="F11" s="22" t="inlineStr">
         <is>
-          <t>If that action isn’t switched on in the backend yet it may quietly do nothing — expected, not a crash.</t>
-        </is>
-      </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>⚠️  Works, watch out</t>
+          <t>There’s no backend action for this yet, so it won’t actually save anything — expected, not a bug.</t>
+        </is>
+      </c>
+      <c r="G11" s="25" t="inlineStr">
+        <is>
+          <t>⛔  Not ready (expected)</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr"/>
@@ -1386,42 +1386,74 @@
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="15" t="inlineStr"/>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>2 · Health score</t>
-        </is>
-      </c>
+    <row r="15" ht="92" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Dashboard shows an honest error if it can’t load</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>Go offline (or block the network), then open or refresh the dashboard.</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>You see an “Unable to load dashboard” card with a Retry button.</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>It must show a clear error — NOT a fake “new account” with zeros. Click Retry when back online.</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>⚠️  Works, watch out</t>
+        </is>
+      </c>
+      <c r="H15" s="23" t="inlineStr"/>
+      <c r="I15" s="21" t="inlineStr"/>
     </row>
     <row r="16" ht="92" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Overview loads</t>
+          <t>Recent activity feed</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>Open Health.</t>
+          <t>Scroll the recent-activity list; use “load more” if shown.</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>You see your overall score and the five areas.</t>
+          <t>Real recent events with real names (e.g. “A signer signed a document”); older items load as you page down.</t>
         </is>
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>A thriving account shows around 90.</t>
+          <t>Nothing yet → an honest empty state.</t>
         </is>
       </c>
       <c r="G16" s="17" t="inlineStr">
@@ -1435,239 +1467,239 @@
     <row r="17" ht="92" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>Open the Financial area</t>
+          <t>Onboarding AI co-founder panel</t>
         </is>
       </c>
       <c r="C17" s="21" t="inlineStr">
         <is>
-          <t>Health → Dimensions → Financial</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>Open the “Financial” area.</t>
+          <t>Fill in the first onboarding steps and watch the side panel.</t>
         </is>
       </c>
       <c r="E17" s="21" t="inlineStr">
         <is>
-          <t>It loads with its details.</t>
+          <t>Once your key details are in, a short AI co-founder calibration message appears.</t>
         </is>
       </c>
       <c r="F17" s="22" t="inlineStr">
         <is>
-          <t>Make sure “Financial” isn’t blank (it’s stored under a different name internally).</t>
-        </is>
-      </c>
-      <c r="G17" s="24" t="inlineStr">
-        <is>
-          <t>⚠️  Works, watch out</t>
+          <t>It shows up once the system has prepared it; brand-new/empty profiles may not show it yet.</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr"/>
       <c r="I17" s="21" t="inlineStr"/>
     </row>
-    <row r="18" ht="92" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>2 · Health score</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="92" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Overview loads</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Open Health.</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>You see your overall score and the five areas.</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>A thriving account shows around 90.</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="inlineStr"/>
+      <c r="I19" s="15" t="inlineStr"/>
+    </row>
+    <row r="20" ht="92" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Open the Financial area</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>Health → Dimensions → Financial</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Open the “Financial” area.</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>It loads with its details.</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>Make sure “Financial” isn’t blank (it’s stored under a different name internally).</t>
+        </is>
+      </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>⚠️  Works, watch out</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr"/>
+      <c r="I20" s="21" t="inlineStr"/>
+    </row>
+    <row r="21" ht="92" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Change the history range</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>Health → Trend history</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Switch the time range (7d / 30d / 90d / all).</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>The chart updates to match the range you picked.</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H18" s="18" t="inlineStr"/>
-      <c r="I18" s="15" t="inlineStr"/>
-    </row>
-    <row r="19" ht="92" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr"/>
+      <c r="I21" s="15" t="inlineStr"/>
+    </row>
+    <row r="22" ht="92" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>Benchmarks</t>
         </is>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C22" s="21" t="inlineStr">
         <is>
           <t>Health → Benchmarks</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>Open Benchmarks.</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E22" s="21" t="inlineStr">
         <is>
           <t>You see comparison data, OR an honest “not enough data yet” message.</t>
         </is>
       </c>
-      <c r="F19" s="22" t="inlineStr">
+      <c r="F22" s="22" t="inlineStr">
         <is>
           <t>If empty it should SAY so — not show made-up numbers.</t>
         </is>
       </c>
-      <c r="G19" s="24" t="inlineStr">
+      <c r="G22" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H19" s="23" t="inlineStr"/>
-      <c r="I19" s="21" t="inlineStr"/>
-    </row>
-    <row r="20" ht="92" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>Accept / dismiss a recommendation</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>Health → Recommendations</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>Accept or dismiss a recommendation.</t>
-        </is>
-      </c>
-      <c r="E20" s="15" t="inlineStr">
-        <is>
-          <t>It resolves and leaves the list.</t>
-        </is>
-      </c>
-      <c r="F20" s="16" t="inlineStr">
-        <is>
-          <t>The main test account may have zero — try a lower-scoring account. Acting on the same one twice may say “already resolved”.</t>
-        </is>
-      </c>
-      <c r="G20" s="24" t="inlineStr">
-        <is>
-          <t>⚠️  Works, watch out</t>
-        </is>
-      </c>
-      <c r="H20" s="18" t="inlineStr"/>
-      <c r="I20" s="15" t="inlineStr"/>
-    </row>
-    <row r="21" ht="92" customHeight="1">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>2.6</t>
-        </is>
-      </c>
-      <c r="B21" s="20" t="inlineStr">
-        <is>
-          <t>Charts show real data</t>
-        </is>
-      </c>
-      <c r="C21" s="21" t="inlineStr">
-        <is>
-          <t>Health → overview, Trend history, a single dimension</t>
-        </is>
-      </c>
-      <c r="D21" s="21" t="inlineStr">
-        <is>
-          <t>Look at the three charts: the “Dimension balance” wheel, the “Score over time” chart, and a dimension’s trend chart.</t>
-        </is>
-      </c>
-      <c r="E21" s="21" t="inlineStr">
-        <is>
-          <t>The wheel shows your five scores; the score-over-time chart has a 0–100 scale and a tooltip; a dimension shows its own trend.</t>
-        </is>
-      </c>
-      <c r="F21" s="22" t="inlineStr">
-        <is>
-          <t>Only one assessment done → the score chart shows a single dot (correct). The dashboard KPI cards no longer show a mini trend line (there’s no real trend data for them).</t>
-        </is>
-      </c>
-      <c r="G21" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H21" s="23" t="inlineStr"/>
-      <c r="I21" s="21" t="inlineStr"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>3 · Today’s Mission</t>
-        </is>
-      </c>
+      <c r="H22" s="23" t="inlineStr"/>
+      <c r="I22" s="21" t="inlineStr"/>
     </row>
     <row r="23" ht="92" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Load today’s mission</t>
+          <t>Accept / dismiss a recommendation</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>Today’s Mission</t>
+          <t>Health → Recommendations</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>Open it.</t>
+          <t>Accept or dismiss a recommendation.</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>You see today’s tasks and your streak.</t>
+          <t>It resolves and leaves the list.</t>
         </is>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
-          <t>A weekend-off day can legitimately have no tasks.</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
+          <t>The main test account may have zero — try a lower-scoring account. Acting on the same one twice may say “already resolved”.</t>
+        </is>
+      </c>
+      <c r="G23" s="24" t="inlineStr">
+        <is>
+          <t>⚠️  Works, watch out</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr"/>
@@ -1676,32 +1708,32 @@
     <row r="24" ht="92" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Task actions</t>
+          <t>Charts show real data</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>Today’s Mission</t>
+          <t>Health → overview, Trend history, a single dimension</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>Complete, snooze, reject, add, or reorder a task.</t>
+          <t>Look at the three charts: the “Dimension balance” wheel, the “Score over time” chart, and a dimension’s trend chart.</t>
         </is>
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>Each updates, and the list and streak refresh correctly.</t>
+          <t>The wheel shows your five scores; the score-over-time chart has a 0–100 scale and a tooltip; a dimension shows its own trend.</t>
         </is>
       </c>
       <c r="F24" s="22" t="inlineStr">
         <is>
-          <t>Completing a task is final — you can’t un-complete it.</t>
+          <t>Only one assessment done → the score chart shows a single dot (correct). The dashboard KPI cards no longer show a mini trend line (there’s no real trend data for them).</t>
         </is>
       </c>
       <c r="G24" s="17" t="inlineStr">
@@ -1712,763 +1744,763 @@
       <c r="H24" s="23" t="inlineStr"/>
       <c r="I24" s="21" t="inlineStr"/>
     </row>
-    <row r="25" ht="92" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>3 · Today’s Mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="92" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Load today’s mission</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>Today’s Mission</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>Open it.</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>You see today’s tasks and your streak.</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>A weekend-off day can legitimately have no tasks.</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr"/>
+      <c r="I26" s="15" t="inlineStr"/>
+    </row>
+    <row r="27" ht="92" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>Task actions</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>Today’s Mission</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="inlineStr">
+        <is>
+          <t>Complete, snooze, reject, add, or reorder a task.</t>
+        </is>
+      </c>
+      <c r="E27" s="21" t="inlineStr">
+        <is>
+          <t>Each updates, and the list and streak refresh correctly.</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>Completing a task is final — you can’t un-complete it.</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H27" s="23" t="inlineStr"/>
+      <c r="I27" s="21" t="inlineStr"/>
+    </row>
+    <row r="28" ht="92" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Reject a task</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>Today’s Mission</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>Reject a task and pick a reason.</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>It’s rejected with the reason you chose.</t>
         </is>
       </c>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>Use the reason chips provided (don’t type your own).</t>
         </is>
       </c>
-      <c r="G25" s="24" t="inlineStr">
+      <c r="G28" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H25" s="18" t="inlineStr"/>
-      <c r="I25" s="15" t="inlineStr"/>
-    </row>
-    <row r="26" ht="92" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="H28" s="18" t="inlineStr"/>
+      <c r="I28" s="15" t="inlineStr"/>
+    </row>
+    <row r="29" ht="92" customHeight="1">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Mission settings</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>Mission → Settings</t>
         </is>
       </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>Change mission size, delivery time, or the weekends option.</t>
         </is>
       </c>
-      <c r="E26" s="21" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>Your settings save.</t>
         </is>
       </c>
-      <c r="F26" s="22" t="inlineStr">
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>Time flips between 12-hour and 24-hour; “weekends off” is the opposite of “weekend missions”.</t>
         </is>
       </c>
-      <c r="G26" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H26" s="23" t="inlineStr"/>
-      <c r="I26" s="21" t="inlineStr"/>
-    </row>
-    <row r="27" ht="92" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr"/>
+      <c r="I29" s="21" t="inlineStr"/>
+    </row>
+    <row r="30" ht="92" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>History pages</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>Mission → Completed / Streaks / Upcoming</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>Open each.</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>They fill with your real history.</t>
         </is>
       </c>
-      <c r="F27" s="16" t="inlineStr">
+      <c r="F30" s="16" t="inlineStr">
         <is>
           <t>No history yet → an honest empty message.</t>
         </is>
       </c>
-      <c r="G27" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H27" s="18" t="inlineStr"/>
-      <c r="I27" s="15" t="inlineStr"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="inlineStr"/>
+      <c r="I30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>4 · Roadmap</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="92" customHeight="1">
-      <c r="A29" s="13" t="inlineStr">
+    <row r="32" ht="92" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>Load the roadmap</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C32" s="15" t="inlineStr">
         <is>
           <t>Roadmap</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="D32" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>You see phases → milestones → tasks.</t>
         </is>
       </c>
-      <c r="F29" s="16" t="inlineStr">
+      <c r="F32" s="16" t="inlineStr">
         <is>
           <t>A “slipped / behind” count shows if any dates have slipped.</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H29" s="18" t="inlineStr"/>
-      <c r="I29" s="15" t="inlineStr"/>
-    </row>
-    <row r="30" ht="92" customHeight="1">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H32" s="18" t="inlineStr"/>
+      <c r="I32" s="15" t="inlineStr"/>
+    </row>
+    <row r="33" ht="92" customHeight="1">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>Add / edit / delete</t>
         </is>
       </c>
-      <c r="C30" s="21" t="inlineStr">
+      <c r="C33" s="21" t="inlineStr">
         <is>
           <t>Roadmap</t>
         </is>
       </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>Add, edit, or delete a phase, milestone or task.</t>
         </is>
       </c>
-      <c r="E30" s="21" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>The change saves and the roadmap updates.</t>
         </is>
       </c>
-      <c r="F30" s="22" t="inlineStr">
+      <c r="F33" s="22" t="inlineStr">
         <is>
           <t>Editors only — a mentor/viewer can’t make changes.</t>
         </is>
       </c>
-      <c r="G30" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr"/>
-      <c r="I30" s="21" t="inlineStr"/>
-    </row>
-    <row r="31" ht="92" customHeight="1">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H33" s="23" t="inlineStr"/>
+      <c r="I33" s="21" t="inlineStr"/>
+    </row>
+    <row r="34" ht="92" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>Block a dependency loop</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C34" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Dependencies</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>Try to link two tasks so they depend on each other in a circle.</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E34" s="15" t="inlineStr">
         <is>
           <t>The app refuses to create the circular link.</t>
         </is>
       </c>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="F34" s="16" t="inlineStr">
         <is>
           <t>It should block the loop.</t>
         </is>
       </c>
-      <c r="G31" s="24" t="inlineStr">
+      <c r="G34" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H31" s="18" t="inlineStr"/>
-      <c r="I31" s="15" t="inlineStr"/>
-    </row>
-    <row r="32" ht="92" customHeight="1">
-      <c r="A32" s="19" t="inlineStr">
+      <c r="H34" s="18" t="inlineStr"/>
+      <c r="I34" s="15" t="inlineStr"/>
+    </row>
+    <row r="35" ht="92" customHeight="1">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>Apply a template</t>
         </is>
       </c>
-      <c r="C32" s="21" t="inlineStr">
+      <c r="C35" s="21" t="inlineStr">
         <is>
           <t>Roadmap → Templates</t>
         </is>
       </c>
-      <c r="D32" s="21" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>Browse the gallery and apply a template.</t>
         </is>
       </c>
-      <c r="E32" s="21" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>The roadmap updates from the template.</t>
         </is>
       </c>
-      <c r="F32" s="22" t="inlineStr">
+      <c r="F35" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr"/>
-      <c r="I32" s="21" t="inlineStr"/>
-    </row>
-    <row r="33" ht="92" customHeight="1">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H35" s="23" t="inlineStr"/>
+      <c r="I35" s="21" t="inlineStr"/>
+    </row>
+    <row r="36" ht="92" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>AI Re-plan — preview &amp; apply</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Re-Plan</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>Preview an AI re-plan, then apply it, and check history.</t>
         </is>
       </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E36" s="15" t="inlineStr">
         <is>
           <t>Preview shows changes; applying updates the plan; history logs it.</t>
         </is>
       </c>
-      <c r="F33" s="16" t="inlineStr">
+      <c r="F36" s="16" t="inlineStr">
         <is>
           <t>Nothing changes until you click Apply.</t>
         </is>
       </c>
-      <c r="G33" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H33" s="18" t="inlineStr"/>
-      <c r="I33" s="15" t="inlineStr"/>
-    </row>
-    <row r="34" ht="92" customHeight="1">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H36" s="18" t="inlineStr"/>
+      <c r="I36" s="15" t="inlineStr"/>
+    </row>
+    <row r="37" ht="92" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>Move a task on the Kanban board</t>
         </is>
       </c>
-      <c r="C34" s="21" t="inlineStr">
+      <c r="C37" s="21" t="inlineStr">
         <is>
           <t>Roadmap → Kanban (Status view)</t>
         </is>
       </c>
-      <c r="D34" s="21" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>Drag a task card between columns (To Do / In Progress / Done).</t>
         </is>
       </c>
-      <c r="E34" s="21" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>The card moves and the change stays after a refresh.</t>
         </is>
       </c>
-      <c r="F34" s="22" t="inlineStr">
+      <c r="F37" s="22" t="inlineStr">
         <is>
           <t>Mentor/viewer → the card snaps back (permission working). The “Phase” view isn’t drag-and-drop; tap a card to open it.</t>
         </is>
       </c>
-      <c r="G34" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H34" s="23" t="inlineStr"/>
-      <c r="I34" s="21" t="inlineStr"/>
-    </row>
-    <row r="35" ht="92" customHeight="1">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H37" s="23" t="inlineStr"/>
+      <c r="I37" s="21" t="inlineStr"/>
+    </row>
+    <row r="38" ht="92" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Re-plan — date changes &amp; history</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C38" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Re-Plan</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>Generate a re-plan; expand a past entry under “Re-plan History”.</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="E38" s="15" t="inlineStr">
         <is>
           <t>Each change shows old date → new date and how far it moved (e.g. “+17 days”); history entries expand to their before/after dates.</t>
         </is>
       </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="F38" s="16" t="inlineStr">
         <is>
           <t>Deltas come from the real dates — nothing invented.</t>
         </is>
       </c>
-      <c r="G35" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H35" s="18" t="inlineStr"/>
-      <c r="I35" s="15" t="inlineStr"/>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H38" s="18" t="inlineStr"/>
+      <c r="I38" s="15" t="inlineStr"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t>5 · Business Builder</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="92" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
+    <row r="40" ht="92" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>Overview</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C40" s="15" t="inlineStr">
         <is>
           <t>Business Builder</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E37" s="15" t="inlineStr">
+      <c r="E40" s="15" t="inlineStr">
         <is>
           <t>You see each canvas with a completion %.</t>
         </is>
       </c>
-      <c r="F37" s="16" t="inlineStr">
+      <c r="F40" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H37" s="18" t="inlineStr"/>
-      <c r="I37" s="15" t="inlineStr"/>
-    </row>
-    <row r="38" ht="92" customHeight="1">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H40" s="18" t="inlineStr"/>
+      <c r="I40" s="15" t="inlineStr"/>
+    </row>
+    <row r="41" ht="92" customHeight="1">
+      <c r="A41" s="19" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B41" s="20" t="inlineStr">
         <is>
           <t>Lean canvas saves</t>
         </is>
       </c>
-      <c r="C38" s="21" t="inlineStr">
+      <c r="C41" s="21" t="inlineStr">
         <is>
           <t>Business Builder → Lean Canvas</t>
         </is>
       </c>
-      <c r="D38" s="21" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>Edit some blocks and wait a moment.</t>
         </is>
       </c>
-      <c r="E38" s="21" t="inlineStr">
+      <c r="E41" s="21" t="inlineStr">
         <is>
           <t>It saves on its own.</t>
         </is>
       </c>
-      <c r="F38" s="22" t="inlineStr">
+      <c r="F41" s="22" t="inlineStr">
         <is>
           <t>Advanced: editing the same canvas in two tabs may briefly show it reconciling — that’s the safety check.</t>
         </is>
       </c>
-      <c r="G38" s="24" t="inlineStr">
+      <c r="G41" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H38" s="23" t="inlineStr"/>
-      <c r="I38" s="21" t="inlineStr"/>
-    </row>
-    <row r="39" ht="92" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="H41" s="23" t="inlineStr"/>
+      <c r="I41" s="21" t="inlineStr"/>
+    </row>
+    <row r="42" ht="92" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>Canvases save automatically</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>Business Model / Value Proposition / SWOT / Mission &amp; Vision</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>Edit and pause.</t>
         </is>
       </c>
-      <c r="E39" s="15" t="inlineStr">
+      <c r="E42" s="15" t="inlineStr">
         <is>
           <t>It saves on its own after you stop typing.</t>
         </is>
       </c>
-      <c r="F39" s="16" t="inlineStr">
+      <c r="F42" s="16" t="inlineStr">
         <is>
           <t>Pause after typing to let it save.</t>
         </is>
       </c>
-      <c r="G39" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H39" s="18" t="inlineStr"/>
-      <c r="I39" s="15" t="inlineStr"/>
-    </row>
-    <row r="40" ht="92" customHeight="1">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H42" s="18" t="inlineStr"/>
+      <c r="I42" s="15" t="inlineStr"/>
+    </row>
+    <row r="43" ht="92" customHeight="1">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="B40" s="20" t="inlineStr">
+      <c r="B43" s="20" t="inlineStr">
         <is>
           <t>Records — add / edit / delete</t>
         </is>
       </c>
-      <c r="C40" s="21" t="inlineStr">
+      <c r="C43" s="21" t="inlineStr">
         <is>
           <t>Personas / Competitive / Pricing / Revenue</t>
         </is>
       </c>
-      <c r="D40" s="21" t="inlineStr">
+      <c r="D43" s="21" t="inlineStr">
         <is>
           <t>Create, edit, and delete a record.</t>
         </is>
       </c>
-      <c r="E40" s="21" t="inlineStr">
+      <c r="E43" s="21" t="inlineStr">
         <is>
           <t>The list updates.</t>
         </is>
       </c>
-      <c r="F40" s="22" t="inlineStr">
+      <c r="F43" s="22" t="inlineStr">
         <is>
           <t>Leaving a required field empty shows a validation message. Pricing has tiers inside it.</t>
         </is>
       </c>
-      <c r="G40" s="24" t="inlineStr">
+      <c r="G43" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H40" s="23" t="inlineStr"/>
-      <c r="I40" s="21" t="inlineStr"/>
-    </row>
-    <row r="41" ht="92" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="H43" s="23" t="inlineStr"/>
+      <c r="I43" s="21" t="inlineStr"/>
+    </row>
+    <row r="44" ht="92" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>Suggestions</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C44" s="15" t="inlineStr">
         <is>
           <t>Business Builder → Suggestions</t>
         </is>
       </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>Approve or reject a suggestion.</t>
         </is>
       </c>
-      <c r="E41" s="15" t="inlineStr">
+      <c r="E44" s="15" t="inlineStr">
         <is>
           <t>It applies or updates.</t>
         </is>
       </c>
-      <c r="F41" s="16" t="inlineStr">
+      <c r="F44" s="16" t="inlineStr">
         <is>
           <t>May say “no longer pending” if the canvas has moved on.</t>
         </is>
       </c>
-      <c r="G41" s="24" t="inlineStr">
+      <c r="G44" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H41" s="18" t="inlineStr"/>
-      <c r="I41" s="15" t="inlineStr"/>
-    </row>
-    <row r="42" ht="92" customHeight="1">
-      <c r="A42" s="19" t="inlineStr">
+      <c r="H44" s="18" t="inlineStr"/>
+      <c r="I44" s="15" t="inlineStr"/>
+    </row>
+    <row r="45" ht="92" customHeight="1">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>5.6</t>
         </is>
       </c>
-      <c r="B42" s="20" t="inlineStr">
+      <c r="B45" s="20" t="inlineStr">
         <is>
           <t>Positioning map</t>
         </is>
       </c>
-      <c r="C42" s="21" t="inlineStr">
+      <c r="C45" s="21" t="inlineStr">
         <is>
           <t>Business Builder → Positioning map</t>
         </is>
       </c>
-      <c r="D42" s="21" t="inlineStr">
+      <c r="D45" s="21" t="inlineStr">
         <is>
           <t>Edit the axes.</t>
         </is>
       </c>
-      <c r="E42" s="21" t="inlineStr">
+      <c r="E45" s="21" t="inlineStr">
         <is>
           <t>Competitors plot against your saved axes.</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F45" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G42" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H42" s="23" t="inlineStr"/>
-      <c r="I42" s="21" t="inlineStr"/>
-    </row>
-    <row r="43" ht="92" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>5.7</t>
-        </is>
-      </c>
-      <c r="B43" s="14" t="inlineStr">
-        <is>
-          <t>AI-fill / AI draft</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
-        <is>
-          <t>Any canvas</t>
-        </is>
-      </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>Click AI-fill / AI draft.</t>
-        </is>
-      </c>
-      <c r="E43" s="15" t="inlineStr">
-        <is>
-          <t>It says “queued — coming soon”.</t>
-        </is>
-      </c>
-      <c r="F43" s="16" t="inlineStr">
-        <is>
-          <t>It never actually finishes yet — expected, not a bug.</t>
-        </is>
-      </c>
-      <c r="G43" s="25" t="inlineStr">
-        <is>
-          <t>⛔  Not ready (expected)</t>
-        </is>
-      </c>
-      <c r="H43" s="18" t="inlineStr"/>
-      <c r="I43" s="15" t="inlineStr"/>
-    </row>
-    <row r="44" ht="92" customHeight="1">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>5.8</t>
-        </is>
-      </c>
-      <c r="B44" s="20" t="inlineStr">
-        <is>
-          <t>Edit &amp; reorder canvas notes</t>
-        </is>
-      </c>
-      <c r="C44" s="21" t="inlineStr">
-        <is>
-          <t>Business Model / Value Proposition / SWOT</t>
-        </is>
-      </c>
-      <c r="D44" s="21" t="inlineStr">
-        <is>
-          <t>Click a note to edit it in place (Enter saves, Esc cancels). Then hover a note, grab its drag handle, and drag it to reorder within the same box.</t>
-        </is>
-      </c>
-      <c r="E44" s="21" t="inlineStr">
-        <is>
-          <t>The note updates and saves; the reordered notes save in the new order.</t>
-        </is>
-      </c>
-      <c r="F44" s="22" t="inlineStr">
-        <is>
-          <t>Emptying a note and pressing Enter deletes it. Reorder stays within one box. “Mission &amp; Vision” is a text box; “Lean Canvas” doesn’t have these yet.</t>
-        </is>
-      </c>
-      <c r="G44" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H44" s="23" t="inlineStr"/>
-      <c r="I44" s="21" t="inlineStr"/>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>6 · Notifications, Journal &amp; Learning</t>
-        </is>
-      </c>
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H45" s="23" t="inlineStr"/>
+      <c r="I45" s="21" t="inlineStr"/>
     </row>
     <row r="46" ht="92" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.7</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Notifications inbox</t>
+          <t>AI-fill / AI draft</t>
         </is>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Bell / Notifications</t>
+          <t>Any canvas</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>Open it, mark one read, and “mark all read”.</t>
+          <t>Click AI-fill / AI draft.</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>The unread count updates.</t>
+          <t>It says “queued — coming soon”.</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G46" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
+          <t>It never actually finishes yet — expected, not a bug.</t>
+        </is>
+      </c>
+      <c r="G46" s="25" t="inlineStr">
+        <is>
+          <t>⛔  Not ready (expected)</t>
         </is>
       </c>
       <c r="H46" s="18" t="inlineStr"/>
@@ -2477,32 +2509,32 @@
     <row r="47" ht="92" customHeight="1">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="B47" s="20" t="inlineStr">
         <is>
-          <t>Email preferences</t>
+          <t>Edit &amp; reorder canvas notes</t>
         </is>
       </c>
       <c r="C47" s="21" t="inlineStr">
         <is>
-          <t>Notifications → Preferences</t>
+          <t>Business Model / Value Proposition / SWOT</t>
         </is>
       </c>
       <c r="D47" s="21" t="inlineStr">
         <is>
-          <t>Toggle the master email switch and the 5 category switches.</t>
+          <t>Click a note to edit it in place (Enter saves, Esc cancels). Then hover a note, grab its drag handle, and drag it to reorder within the same box.</t>
         </is>
       </c>
       <c r="E47" s="21" t="inlineStr">
         <is>
-          <t>They save.</t>
+          <t>The note updates and saves; the reordered notes save in the new order.</t>
         </is>
       </c>
       <c r="F47" s="22" t="inlineStr">
         <is>
-          <t>The “Digest &amp; quiet hours” and “Announcements” tabs are demo-only for now.</t>
+          <t>Emptying a note and pressing Enter deletes it. Reorder stays within one box. “Mission &amp; Vision” is a text box; “Lean Canvas” doesn’t have these yet.</t>
         </is>
       </c>
       <c r="G47" s="17" t="inlineStr">
@@ -2516,32 +2548,32 @@
     <row r="48" ht="92" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>5.9</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Read the journal</t>
+          <t>AI budget guardrail</t>
         </is>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>Any canvas (AI draft) + the AI usage display</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>Read journal entries.</t>
+          <t>Look at the AI-draft buttons and the AI usage display.</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>Reading works.</t>
+          <t>When the workspace is over its daily AI budget, AI-draft buttons show “AI draft paused (until …)” instead of running; the usage display shows tokens used, or “Unlimited” when there’s no cap.</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Honest pause — it never pretends to produce an AI result it can’t.</t>
         </is>
       </c>
       <c r="G48" s="17" t="inlineStr">
@@ -2552,69 +2584,37 @@
       <c r="H48" s="18" t="inlineStr"/>
       <c r="I48" s="15" t="inlineStr"/>
     </row>
-    <row r="49" ht="92" customHeight="1">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>6.4</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="inlineStr">
-        <is>
-          <t>Save a new journal entry</t>
-        </is>
-      </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>Journal</t>
-        </is>
-      </c>
-      <c r="D49" s="21" t="inlineStr">
-        <is>
-          <t>Try to save a new entry.</t>
-        </is>
-      </c>
-      <c r="E49" s="21" t="inlineStr">
-        <is>
-          <t>It fails gracefully — it doesn’t crash the page.</t>
-        </is>
-      </c>
-      <c r="F49" s="22" t="inlineStr">
-        <is>
-          <t>Saving isn’t set up on the test server yet — expected to fail softly.</t>
-        </is>
-      </c>
-      <c r="G49" s="25" t="inlineStr">
-        <is>
-          <t>⛔  Not ready (expected)</t>
-        </is>
-      </c>
-      <c r="H49" s="23" t="inlineStr"/>
-      <c r="I49" s="21" t="inlineStr"/>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>6 · Notifications, Journal &amp; Learning</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="92" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Learning academy</t>
+          <t>Notifications inbox</t>
         </is>
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Academy</t>
+          <t>Bell / Notifications</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>Browse courses / articles / paths / certificates, enroll, and complete a lesson.</t>
+          <t>Open it, mark one read, and “mark all read”.</t>
         </is>
       </c>
       <c r="E50" s="15" t="inlineStr">
         <is>
-          <t>These work and save.</t>
+          <t>The unread count updates.</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
@@ -2630,37 +2630,69 @@
       <c r="H50" s="18" t="inlineStr"/>
       <c r="I50" s="15" t="inlineStr"/>
     </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
-        <is>
-          <t>7 · Documents</t>
-        </is>
-      </c>
+    <row r="51" ht="92" customHeight="1">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>Email preferences</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>Notifications → Preferences</t>
+        </is>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>Toggle the master email switch and the 5 category switches.</t>
+        </is>
+      </c>
+      <c r="E51" s="21" t="inlineStr">
+        <is>
+          <t>They save.</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr">
+        <is>
+          <t>The “Digest &amp; quiet hours” and “Announcements” tabs are demo-only for now.</t>
+        </is>
+      </c>
+      <c r="G51" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H51" s="23" t="inlineStr"/>
+      <c r="I51" s="21" t="inlineStr"/>
     </row>
     <row r="52" ht="92" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Files</t>
+          <t>Read the journal</t>
         </is>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
         <is>
-          <t>Upload, list, and delete a file.</t>
+          <t>Read journal entries.</t>
         </is>
       </c>
       <c r="E52" s="15" t="inlineStr">
         <is>
-          <t>All three work.</t>
+          <t>Reading works.</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
@@ -2679,37 +2711,37 @@
     <row r="53" ht="92" customHeight="1">
       <c r="A53" s="19" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B53" s="20" t="inlineStr">
         <is>
-          <t>Share a document</t>
+          <t>Save a new journal entry</t>
         </is>
       </c>
       <c r="C53" s="21" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>Journal</t>
         </is>
       </c>
       <c r="D53" s="21" t="inlineStr">
         <is>
-          <t>Share a document, then remove the share.</t>
+          <t>Try to save a new entry.</t>
         </is>
       </c>
       <c r="E53" s="21" t="inlineStr">
         <is>
-          <t>The share list updates.</t>
+          <t>It fails gracefully — it doesn’t crash the page.</t>
         </is>
       </c>
       <c r="F53" s="22" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G53" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
+          <t>Saving isn’t set up on the test server yet — expected to fail softly.</t>
+        </is>
+      </c>
+      <c r="G53" s="25" t="inlineStr">
+        <is>
+          <t>⛔  Not ready (expected)</t>
         </is>
       </c>
       <c r="H53" s="23" t="inlineStr"/>
@@ -2718,27 +2750,27 @@
     <row r="54" ht="92" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Signature requests</t>
+          <t>Learning academy</t>
         </is>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Documents → Signatures</t>
+          <t>Academy</t>
         </is>
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>Send, remind, or cancel a signature request.</t>
+          <t>Browse courses / articles / paths / certificates, enroll, and complete a lesson.</t>
         </is>
       </c>
       <c r="E54" s="15" t="inlineStr">
         <is>
-          <t>The status reflects what you did.</t>
+          <t>These work and save.</t>
         </is>
       </c>
       <c r="F54" s="16" t="inlineStr">
@@ -2754,79 +2786,47 @@
       <c r="H54" s="18" t="inlineStr"/>
       <c r="I54" s="15" t="inlineStr"/>
     </row>
-    <row r="55" ht="92" customHeight="1">
-      <c r="A55" s="19" t="inlineStr">
-        <is>
-          <t>7.4</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="inlineStr">
-        <is>
-          <t>Create from a template</t>
-        </is>
-      </c>
-      <c r="C55" s="21" t="inlineStr">
-        <is>
-          <t>Documents → Templates</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="inlineStr">
-        <is>
-          <t>Create a document from a template.</t>
-        </is>
-      </c>
-      <c r="E55" s="21" t="inlineStr">
-        <is>
-          <t>It creates the document.</t>
-        </is>
-      </c>
-      <c r="F55" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G55" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H55" s="23" t="inlineStr"/>
-      <c r="I55" s="21" t="inlineStr"/>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>7 · Documents</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="92" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Edit &amp; save a document</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Documents → open a document</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="D56" s="15" t="inlineStr">
         <is>
-          <t>Open the editor, make edits, and save.</t>
+          <t>Upload, list, and delete a file.</t>
         </is>
       </c>
       <c r="E56" s="15" t="inlineStr">
         <is>
-          <t>Your edits save.</t>
+          <t>All three work.</t>
         </is>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
-          <t>Documents don’t auto-save — click Save. If it was changed elsewhere you get a “reload” banner and it won’t overwrite.</t>
-        </is>
-      </c>
-      <c r="G56" s="24" t="inlineStr">
-        <is>
-          <t>⚠️  Works, watch out</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
         </is>
       </c>
       <c r="H56" s="18" t="inlineStr"/>
@@ -2835,37 +2835,37 @@
     <row r="57" ht="92" customHeight="1">
       <c r="A57" s="19" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B57" s="20" t="inlineStr">
         <is>
-          <t>Open a real emailed sign/share link</t>
+          <t>Share a document</t>
         </is>
       </c>
       <c r="C57" s="21" t="inlineStr">
         <is>
-          <t>The sign/share link</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="D57" s="21" t="inlineStr">
         <is>
-          <t>Open a real emailed link.</t>
+          <t>Share a document, then remove the share.</t>
         </is>
       </c>
       <c r="E57" s="21" t="inlineStr">
         <is>
-          <t>The recipient page works when opened on the app website.</t>
+          <t>The share list updates.</t>
         </is>
       </c>
       <c r="F57" s="22" t="inlineStr">
         <is>
-          <t>Straight from an email it may show a raw data page — open it on the app website instead.</t>
-        </is>
-      </c>
-      <c r="G57" s="25" t="inlineStr">
-        <is>
-          <t>⛔  Not ready (expected)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
         </is>
       </c>
       <c r="H57" s="23" t="inlineStr"/>
@@ -2874,32 +2874,32 @@
     <row r="58" ht="92" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>7.7</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Edit a document’s sections</t>
+          <t>Signature requests</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Documents → open a document</t>
+          <t>Documents → Signatures</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
         <is>
-          <t>Add a section, delete one, drag a section to reorder (or use the up/down arrows), and rename a heading. Then Save.</t>
+          <t>Send, remind, or cancel a signature request.</t>
         </is>
       </c>
       <c r="E58" s="15" t="inlineStr">
         <is>
-          <t>All the section changes save after you click Save.</t>
+          <t>The status reflects what you did.</t>
         </is>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
-          <t>Documents don’t auto-save — you must click Save. Headings used to be read-only.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G58" s="17" t="inlineStr">
@@ -2913,32 +2913,32 @@
     <row r="59" ht="92" customHeight="1">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>7.8</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B59" s="20" t="inlineStr">
         <is>
-          <t>Sign a document</t>
+          <t>Create from a template</t>
         </is>
       </c>
       <c r="C59" s="21" t="inlineStr">
         <is>
-          <t>The signing link, on the app website</t>
+          <t>Documents → Templates</t>
         </is>
       </c>
       <c r="D59" s="21" t="inlineStr">
         <is>
-          <t>Read the preview, type your full name (shown styled like a signature), tick the “I agree…” box, then Sign.</t>
+          <t>Create a document from a template.</t>
         </is>
       </c>
       <c r="E59" s="21" t="inlineStr">
         <is>
-          <t>Your typed name is accepted and you see a “signed — thank you” confirmation.</t>
+          <t>It creates the document.</t>
         </is>
       </c>
       <c r="F59" s="22" t="inlineStr">
         <is>
-          <t>It’s a typed signature (no drawing pad). The Sign button stays disabled until you tick consent.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G59" s="17" t="inlineStr">
@@ -2949,19 +2949,175 @@
       <c r="H59" s="23" t="inlineStr"/>
       <c r="I59" s="21" t="inlineStr"/>
     </row>
+    <row r="60" ht="92" customHeight="1">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>Edit &amp; save a document</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>Documents → open a document</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>Open the editor, make edits, and save.</t>
+        </is>
+      </c>
+      <c r="E60" s="15" t="inlineStr">
+        <is>
+          <t>Your edits save.</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>Documents don’t auto-save — click Save. If it was changed elsewhere you get a “reload” banner and it won’t overwrite.</t>
+        </is>
+      </c>
+      <c r="G60" s="24" t="inlineStr">
+        <is>
+          <t>⚠️  Works, watch out</t>
+        </is>
+      </c>
+      <c r="H60" s="18" t="inlineStr"/>
+      <c r="I60" s="15" t="inlineStr"/>
+    </row>
+    <row r="61" ht="92" customHeight="1">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>7.6</t>
+        </is>
+      </c>
+      <c r="B61" s="20" t="inlineStr">
+        <is>
+          <t>Open a real emailed sign/share link</t>
+        </is>
+      </c>
+      <c r="C61" s="21" t="inlineStr">
+        <is>
+          <t>The sign/share link</t>
+        </is>
+      </c>
+      <c r="D61" s="21" t="inlineStr">
+        <is>
+          <t>Open a real emailed link.</t>
+        </is>
+      </c>
+      <c r="E61" s="21" t="inlineStr">
+        <is>
+          <t>The recipient page works when opened on the app website.</t>
+        </is>
+      </c>
+      <c r="F61" s="22" t="inlineStr">
+        <is>
+          <t>Straight from an email it may show a raw data page — open it on the app website instead.</t>
+        </is>
+      </c>
+      <c r="G61" s="25" t="inlineStr">
+        <is>
+          <t>⛔  Not ready (expected)</t>
+        </is>
+      </c>
+      <c r="H61" s="23" t="inlineStr"/>
+      <c r="I61" s="21" t="inlineStr"/>
+    </row>
+    <row r="62" ht="92" customHeight="1">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Edit a document’s sections</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>Documents → open a document</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>Add a section, delete one, drag a section to reorder (or use the up/down arrows), and rename a heading. Then Save.</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="inlineStr">
+        <is>
+          <t>All the section changes save after you click Save.</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>Documents don’t auto-save — you must click Save. Headings used to be read-only.</t>
+        </is>
+      </c>
+      <c r="G62" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H62" s="18" t="inlineStr"/>
+      <c r="I62" s="15" t="inlineStr"/>
+    </row>
+    <row r="63" ht="92" customHeight="1">
+      <c r="A63" s="19" t="inlineStr">
+        <is>
+          <t>7.8</t>
+        </is>
+      </c>
+      <c r="B63" s="20" t="inlineStr">
+        <is>
+          <t>Sign a document</t>
+        </is>
+      </c>
+      <c r="C63" s="21" t="inlineStr">
+        <is>
+          <t>The signing link, on the app website</t>
+        </is>
+      </c>
+      <c r="D63" s="21" t="inlineStr">
+        <is>
+          <t>Read the preview, type your full name (shown styled like a signature), tick the “I agree…” box, then Sign.</t>
+        </is>
+      </c>
+      <c r="E63" s="21" t="inlineStr">
+        <is>
+          <t>Your typed name is accepted and you see a “signed — thank you” confirmation.</t>
+        </is>
+      </c>
+      <c r="F63" s="22" t="inlineStr">
+        <is>
+          <t>It’s a typed signature (no drawing pad). The Sign button stays disabled until you tick consent.</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H63" s="23" t="inlineStr"/>
+      <c r="I63" s="21" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A51:I51"/>
-    <mergeCell ref="A28:I28"/>
-    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A49:I49"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A31:I31"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A39:I39"/>
+    <mergeCell ref="A55:I55"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
+    <dataValidation sqref="H4:H63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2975,7 +3131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3064,10 +3220,22 @@
     <row r="9" ht="50" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
+          <t>Dashboard briefing “Do it”</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>The “Do it” button on the AI briefing acknowledges locally but can’t save anything — there’s no backend action for it yet (test 1.8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
           <t>Demo-only areas (placeholder data)</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Not connected to real data yet — don’t test as real: Marketing, Sales, Finance, Validation, Funding, Investor Readiness, Legal &amp; Compliance, Calendar, Analytics &amp; Reports, Marketplace, Admin / Super-Admin, and the Notifications “Digest / quiet hours” &amp; “Announcements” tabs.</t>
         </is>

</xml_diff>

<commit_message>
Fix public hero copy and wire sidebar to real workspace identity
- Drop the "AI" qualifier from marketing copy site-wide ("operating
  system", "advisors") across the hero badge/subhead, footer tagline,
  SEO/OG descriptions and nav; add the hero tagline "Built for founders
  at every stage, ..." (comma, no em dash per the house-style guard)
- Wire the sidebar workspace switcher and founder profile to real
  GET /onboarding/state via a new useStartupProfile hook (name, stage,
  logo, founder name/role) instead of the hardcoded Kolo / Amara Okafor
  placeholders; honest null fallbacks, logo img with letter fallback
- Docs: SOP module-35, frontend checklist, QA checklist + regenerated
  xlsx (new case 1.15)
</commit_message>
<xml_diff>
--- a/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
+++ b/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
@@ -882,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1503,1621 +1503,1660 @@
       <c r="H17" s="23" t="inlineStr"/>
       <c r="I17" s="21" t="inlineStr"/>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="18" ht="92" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Sidebar shows your real workspace and name</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Left sidebar (any dashboard page)</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Look at the workspace box at the top of the left sidebar and your profile at the very bottom.</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Both show YOUR real details: your startup name, stage and uploaded logo at the top; your name and role at the bottom.</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>It must NOT show a fixed placeholder like “Kolo” / “Validation stage” or “Amara Okafor” / “Founder” for everyone. A different account should show its own name and logo. No logo yet shows the first letter of the name.</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr"/>
+      <c r="I18" s="15" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>2 · Health score</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="92" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="20" ht="92" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Overview loads</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>Open Health.</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>You see your overall score and the five areas.</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>A thriving account shows around 90.</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H19" s="18" t="inlineStr"/>
-      <c r="I19" s="15" t="inlineStr"/>
-    </row>
-    <row r="20" ht="92" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr"/>
+      <c r="I20" s="15" t="inlineStr"/>
+    </row>
+    <row r="21" ht="92" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>Open the Financial area</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>Health → Dimensions → Financial</t>
         </is>
       </c>
-      <c r="D20" s="21" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>Open the “Financial” area.</t>
         </is>
       </c>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>It loads with its details.</t>
         </is>
       </c>
-      <c r="F20" s="22" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>Make sure “Financial” isn’t blank (it’s stored under a different name internally).</t>
         </is>
       </c>
-      <c r="G20" s="24" t="inlineStr">
+      <c r="G21" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H20" s="23" t="inlineStr"/>
-      <c r="I20" s="21" t="inlineStr"/>
-    </row>
-    <row r="21" ht="92" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="H21" s="23" t="inlineStr"/>
+      <c r="I21" s="21" t="inlineStr"/>
+    </row>
+    <row r="22" ht="92" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Change the history range</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>Health → Trend history</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>Switch the time range (7d / 30d / 90d / all).</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>The chart updates to match the range you picked.</t>
         </is>
       </c>
-      <c r="F21" s="16" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H21" s="18" t="inlineStr"/>
-      <c r="I21" s="15" t="inlineStr"/>
-    </row>
-    <row r="22" ht="92" customHeight="1">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr"/>
+      <c r="I22" s="15" t="inlineStr"/>
+    </row>
+    <row r="23" ht="92" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>Benchmarks</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>Health → Benchmarks</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>Open Benchmarks.</t>
         </is>
       </c>
-      <c r="E22" s="21" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>You see comparison data, OR an honest “not enough data yet” message.</t>
         </is>
       </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="F23" s="22" t="inlineStr">
         <is>
           <t>If empty it should SAY so — not show made-up numbers.</t>
         </is>
       </c>
-      <c r="G22" s="24" t="inlineStr">
+      <c r="G23" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H22" s="23" t="inlineStr"/>
-      <c r="I22" s="21" t="inlineStr"/>
-    </row>
-    <row r="23" ht="92" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="H23" s="23" t="inlineStr"/>
+      <c r="I23" s="21" t="inlineStr"/>
+    </row>
+    <row r="24" ht="92" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Accept / dismiss a recommendation</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>Health → Recommendations</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Accept or dismiss a recommendation.</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>It resolves and leaves the list.</t>
         </is>
       </c>
-      <c r="F23" s="16" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>The main test account may have zero — try a lower-scoring account. Acting on the same one twice may say “already resolved”.</t>
         </is>
       </c>
-      <c r="G23" s="24" t="inlineStr">
+      <c r="G24" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H23" s="18" t="inlineStr"/>
-      <c r="I23" s="15" t="inlineStr"/>
-    </row>
-    <row r="24" ht="92" customHeight="1">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="H24" s="18" t="inlineStr"/>
+      <c r="I24" s="15" t="inlineStr"/>
+    </row>
+    <row r="25" ht="92" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>Charts show real data</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>Health → overview, Trend history, a single dimension</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Look at the three charts: the “Dimension balance” wheel, the “Score over time” chart, and a dimension’s trend chart.</t>
         </is>
       </c>
-      <c r="E24" s="21" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>The wheel shows your five scores; the score-over-time chart has a 0–100 scale and a tooltip; a dimension shows its own trend.</t>
         </is>
       </c>
-      <c r="F24" s="22" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>Only one assessment done → the score chart shows a single dot (correct). The dashboard KPI cards no longer show a mini trend line (there’s no real trend data for them).</t>
         </is>
       </c>
-      <c r="G24" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H24" s="23" t="inlineStr"/>
-      <c r="I24" s="21" t="inlineStr"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H25" s="23" t="inlineStr"/>
+      <c r="I25" s="21" t="inlineStr"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>3 · Today’s Mission</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="92" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="27" ht="92" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Load today’s mission</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>Today’s Mission</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>You see today’s tasks and your streak.</t>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>A weekend-off day can legitimately have no tasks.</t>
         </is>
       </c>
-      <c r="G26" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H26" s="18" t="inlineStr"/>
-      <c r="I26" s="15" t="inlineStr"/>
-    </row>
-    <row r="27" ht="92" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="inlineStr"/>
+      <c r="I27" s="15" t="inlineStr"/>
+    </row>
+    <row r="28" ht="92" customHeight="1">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>Task actions</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>Today’s Mission</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>Complete, snooze, reject, add, or reorder a task.</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>Each updates, and the list and streak refresh correctly.</t>
         </is>
       </c>
-      <c r="F27" s="22" t="inlineStr">
+      <c r="F28" s="22" t="inlineStr">
         <is>
           <t>Completing a task is final — you can’t un-complete it.</t>
         </is>
       </c>
-      <c r="G27" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H27" s="23" t="inlineStr"/>
-      <c r="I27" s="21" t="inlineStr"/>
-    </row>
-    <row r="28" ht="92" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H28" s="23" t="inlineStr"/>
+      <c r="I28" s="21" t="inlineStr"/>
+    </row>
+    <row r="29" ht="92" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Reject a task</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>Today’s Mission</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>Reject a task and pick a reason.</t>
         </is>
       </c>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>It’s rejected with the reason you chose.</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F29" s="16" t="inlineStr">
         <is>
           <t>Use the reason chips provided (don’t type your own).</t>
         </is>
       </c>
-      <c r="G28" s="24" t="inlineStr">
+      <c r="G29" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H28" s="18" t="inlineStr"/>
-      <c r="I28" s="15" t="inlineStr"/>
-    </row>
-    <row r="29" ht="92" customHeight="1">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="H29" s="18" t="inlineStr"/>
+      <c r="I29" s="15" t="inlineStr"/>
+    </row>
+    <row r="30" ht="92" customHeight="1">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>Mission settings</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>Mission → Settings</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>Change mission size, delivery time, or the weekends option.</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>Your settings save.</t>
         </is>
       </c>
-      <c r="F29" s="22" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>Time flips between 12-hour and 24-hour; “weekends off” is the opposite of “weekend missions”.</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H29" s="23" t="inlineStr"/>
-      <c r="I29" s="21" t="inlineStr"/>
-    </row>
-    <row r="30" ht="92" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H30" s="23" t="inlineStr"/>
+      <c r="I30" s="21" t="inlineStr"/>
+    </row>
+    <row r="31" ht="92" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>History pages</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>Mission → Completed / Streaks / Upcoming</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>Open each.</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>They fill with your real history.</t>
         </is>
       </c>
-      <c r="F30" s="16" t="inlineStr">
+      <c r="F31" s="16" t="inlineStr">
         <is>
           <t>No history yet → an honest empty message.</t>
         </is>
       </c>
-      <c r="G30" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H30" s="18" t="inlineStr"/>
-      <c r="I30" s="15" t="inlineStr"/>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H31" s="18" t="inlineStr"/>
+      <c r="I31" s="15" t="inlineStr"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>4 · Roadmap</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="92" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
+    <row r="33" ht="92" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Load the roadmap</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>Roadmap</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>You see phases → milestones → tasks.</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="F33" s="16" t="inlineStr">
         <is>
           <t>A “slipped / behind” count shows if any dates have slipped.</t>
         </is>
       </c>
-      <c r="G32" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H32" s="18" t="inlineStr"/>
-      <c r="I32" s="15" t="inlineStr"/>
-    </row>
-    <row r="33" ht="92" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H33" s="18" t="inlineStr"/>
+      <c r="I33" s="15" t="inlineStr"/>
+    </row>
+    <row r="34" ht="92" customHeight="1">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>Add / edit / delete</t>
         </is>
       </c>
-      <c r="C33" s="21" t="inlineStr">
+      <c r="C34" s="21" t="inlineStr">
         <is>
           <t>Roadmap</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>Add, edit, or delete a phase, milestone or task.</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>The change saves and the roadmap updates.</t>
         </is>
       </c>
-      <c r="F33" s="22" t="inlineStr">
+      <c r="F34" s="22" t="inlineStr">
         <is>
           <t>Editors only — a mentor/viewer can’t make changes.</t>
         </is>
       </c>
-      <c r="G33" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H33" s="23" t="inlineStr"/>
-      <c r="I33" s="21" t="inlineStr"/>
-    </row>
-    <row r="34" ht="92" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H34" s="23" t="inlineStr"/>
+      <c r="I34" s="21" t="inlineStr"/>
+    </row>
+    <row r="35" ht="92" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>Block a dependency loop</t>
         </is>
       </c>
-      <c r="C34" s="15" t="inlineStr">
+      <c r="C35" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Dependencies</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>Try to link two tasks so they depend on each other in a circle.</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="E35" s="15" t="inlineStr">
         <is>
           <t>The app refuses to create the circular link.</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>It should block the loop.</t>
         </is>
       </c>
-      <c r="G34" s="24" t="inlineStr">
+      <c r="G35" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H34" s="18" t="inlineStr"/>
-      <c r="I34" s="15" t="inlineStr"/>
-    </row>
-    <row r="35" ht="92" customHeight="1">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="H35" s="18" t="inlineStr"/>
+      <c r="I35" s="15" t="inlineStr"/>
+    </row>
+    <row r="36" ht="92" customHeight="1">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>Apply a template</t>
         </is>
       </c>
-      <c r="C35" s="21" t="inlineStr">
+      <c r="C36" s="21" t="inlineStr">
         <is>
           <t>Roadmap → Templates</t>
         </is>
       </c>
-      <c r="D35" s="21" t="inlineStr">
+      <c r="D36" s="21" t="inlineStr">
         <is>
           <t>Browse the gallery and apply a template.</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>The roadmap updates from the template.</t>
         </is>
       </c>
-      <c r="F35" s="22" t="inlineStr">
+      <c r="F36" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G35" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H35" s="23" t="inlineStr"/>
-      <c r="I35" s="21" t="inlineStr"/>
-    </row>
-    <row r="36" ht="92" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H36" s="23" t="inlineStr"/>
+      <c r="I36" s="21" t="inlineStr"/>
+    </row>
+    <row r="37" ht="92" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>AI Re-plan — preview &amp; apply</t>
         </is>
       </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Re-Plan</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>Preview an AI re-plan, then apply it, and check history.</t>
         </is>
       </c>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="E37" s="15" t="inlineStr">
         <is>
           <t>Preview shows changes; applying updates the plan; history logs it.</t>
         </is>
       </c>
-      <c r="F36" s="16" t="inlineStr">
+      <c r="F37" s="16" t="inlineStr">
         <is>
           <t>Nothing changes until you click Apply.</t>
         </is>
       </c>
-      <c r="G36" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H36" s="18" t="inlineStr"/>
-      <c r="I36" s="15" t="inlineStr"/>
-    </row>
-    <row r="37" ht="92" customHeight="1">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H37" s="18" t="inlineStr"/>
+      <c r="I37" s="15" t="inlineStr"/>
+    </row>
+    <row r="38" ht="92" customHeight="1">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>Move a task on the Kanban board</t>
         </is>
       </c>
-      <c r="C37" s="21" t="inlineStr">
+      <c r="C38" s="21" t="inlineStr">
         <is>
           <t>Roadmap → Kanban (Status view)</t>
         </is>
       </c>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>Drag a task card between columns (To Do / In Progress / Done).</t>
         </is>
       </c>
-      <c r="E37" s="21" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>The card moves and the change stays after a refresh.</t>
         </is>
       </c>
-      <c r="F37" s="22" t="inlineStr">
+      <c r="F38" s="22" t="inlineStr">
         <is>
           <t>Mentor/viewer → the card snaps back (permission working). The “Phase” view isn’t drag-and-drop; tap a card to open it.</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H37" s="23" t="inlineStr"/>
-      <c r="I37" s="21" t="inlineStr"/>
-    </row>
-    <row r="38" ht="92" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H38" s="23" t="inlineStr"/>
+      <c r="I38" s="21" t="inlineStr"/>
+    </row>
+    <row r="39" ht="92" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>Re-plan — date changes &amp; history</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Re-Plan</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>Generate a re-plan; expand a past entry under “Re-plan History”.</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
+      <c r="E39" s="15" t="inlineStr">
         <is>
           <t>Each change shows old date → new date and how far it moved (e.g. “+17 days”); history entries expand to their before/after dates.</t>
         </is>
       </c>
-      <c r="F38" s="16" t="inlineStr">
+      <c r="F39" s="16" t="inlineStr">
         <is>
           <t>Deltas come from the real dates — nothing invented.</t>
         </is>
       </c>
-      <c r="G38" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H38" s="18" t="inlineStr"/>
-      <c r="I38" s="15" t="inlineStr"/>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="12" t="inlineStr">
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H39" s="18" t="inlineStr"/>
+      <c r="I39" s="15" t="inlineStr"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>5 · Business Builder</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="92" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+    <row r="41" ht="92" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>Overview</t>
         </is>
       </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>Business Builder</t>
         </is>
       </c>
-      <c r="D40" s="15" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E40" s="15" t="inlineStr">
+      <c r="E41" s="15" t="inlineStr">
         <is>
           <t>You see each canvas with a completion %.</t>
         </is>
       </c>
-      <c r="F40" s="16" t="inlineStr">
+      <c r="F41" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H40" s="18" t="inlineStr"/>
-      <c r="I40" s="15" t="inlineStr"/>
-    </row>
-    <row r="41" ht="92" customHeight="1">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H41" s="18" t="inlineStr"/>
+      <c r="I41" s="15" t="inlineStr"/>
+    </row>
+    <row r="42" ht="92" customHeight="1">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>Lean canvas saves</t>
         </is>
       </c>
-      <c r="C41" s="21" t="inlineStr">
+      <c r="C42" s="21" t="inlineStr">
         <is>
           <t>Business Builder → Lean Canvas</t>
         </is>
       </c>
-      <c r="D41" s="21" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>Edit some blocks and wait a moment.</t>
         </is>
       </c>
-      <c r="E41" s="21" t="inlineStr">
+      <c r="E42" s="21" t="inlineStr">
         <is>
           <t>It saves on its own.</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F42" s="22" t="inlineStr">
         <is>
           <t>Advanced: editing the same canvas in two tabs may briefly show it reconciling — that’s the safety check.</t>
         </is>
       </c>
-      <c r="G41" s="24" t="inlineStr">
+      <c r="G42" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H41" s="23" t="inlineStr"/>
-      <c r="I41" s="21" t="inlineStr"/>
-    </row>
-    <row r="42" ht="92" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="H42" s="23" t="inlineStr"/>
+      <c r="I42" s="21" t="inlineStr"/>
+    </row>
+    <row r="43" ht="92" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Canvases save automatically</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>Business Model / Value Proposition / SWOT / Mission &amp; Vision</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>Edit and pause.</t>
         </is>
       </c>
-      <c r="E42" s="15" t="inlineStr">
+      <c r="E43" s="15" t="inlineStr">
         <is>
           <t>It saves on its own after you stop typing.</t>
         </is>
       </c>
-      <c r="F42" s="16" t="inlineStr">
+      <c r="F43" s="16" t="inlineStr">
         <is>
           <t>Pause after typing to let it save.</t>
         </is>
       </c>
-      <c r="G42" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H42" s="18" t="inlineStr"/>
-      <c r="I42" s="15" t="inlineStr"/>
-    </row>
-    <row r="43" ht="92" customHeight="1">
-      <c r="A43" s="19" t="inlineStr">
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H43" s="18" t="inlineStr"/>
+      <c r="I43" s="15" t="inlineStr"/>
+    </row>
+    <row r="44" ht="92" customHeight="1">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="B43" s="20" t="inlineStr">
+      <c r="B44" s="20" t="inlineStr">
         <is>
           <t>Records — add / edit / delete</t>
         </is>
       </c>
-      <c r="C43" s="21" t="inlineStr">
+      <c r="C44" s="21" t="inlineStr">
         <is>
           <t>Personas / Competitive / Pricing / Revenue</t>
         </is>
       </c>
-      <c r="D43" s="21" t="inlineStr">
+      <c r="D44" s="21" t="inlineStr">
         <is>
           <t>Create, edit, and delete a record.</t>
         </is>
       </c>
-      <c r="E43" s="21" t="inlineStr">
+      <c r="E44" s="21" t="inlineStr">
         <is>
           <t>The list updates.</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F44" s="22" t="inlineStr">
         <is>
           <t>Leaving a required field empty shows a validation message. Pricing has tiers inside it.</t>
         </is>
       </c>
-      <c r="G43" s="24" t="inlineStr">
+      <c r="G44" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H43" s="23" t="inlineStr"/>
-      <c r="I43" s="21" t="inlineStr"/>
-    </row>
-    <row r="44" ht="92" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="H44" s="23" t="inlineStr"/>
+      <c r="I44" s="21" t="inlineStr"/>
+    </row>
+    <row r="45" ht="92" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>Suggestions</t>
         </is>
       </c>
-      <c r="C44" s="15" t="inlineStr">
+      <c r="C45" s="15" t="inlineStr">
         <is>
           <t>Business Builder → Suggestions</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D45" s="15" t="inlineStr">
         <is>
           <t>Approve or reject a suggestion.</t>
         </is>
       </c>
-      <c r="E44" s="15" t="inlineStr">
+      <c r="E45" s="15" t="inlineStr">
         <is>
           <t>It applies or updates.</t>
         </is>
       </c>
-      <c r="F44" s="16" t="inlineStr">
+      <c r="F45" s="16" t="inlineStr">
         <is>
           <t>May say “no longer pending” if the canvas has moved on.</t>
         </is>
       </c>
-      <c r="G44" s="24" t="inlineStr">
+      <c r="G45" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H44" s="18" t="inlineStr"/>
-      <c r="I44" s="15" t="inlineStr"/>
-    </row>
-    <row r="45" ht="92" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="H45" s="18" t="inlineStr"/>
+      <c r="I45" s="15" t="inlineStr"/>
+    </row>
+    <row r="46" ht="92" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>5.6</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>Positioning map</t>
         </is>
       </c>
-      <c r="C45" s="21" t="inlineStr">
+      <c r="C46" s="21" t="inlineStr">
         <is>
           <t>Business Builder → Positioning map</t>
         </is>
       </c>
-      <c r="D45" s="21" t="inlineStr">
+      <c r="D46" s="21" t="inlineStr">
         <is>
           <t>Edit the axes.</t>
         </is>
       </c>
-      <c r="E45" s="21" t="inlineStr">
+      <c r="E46" s="21" t="inlineStr">
         <is>
           <t>Competitors plot against your saved axes.</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F46" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G45" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H45" s="23" t="inlineStr"/>
-      <c r="I45" s="21" t="inlineStr"/>
-    </row>
-    <row r="46" ht="92" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="G46" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H46" s="23" t="inlineStr"/>
+      <c r="I46" s="21" t="inlineStr"/>
+    </row>
+    <row r="47" ht="92" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>5.7</t>
         </is>
       </c>
-      <c r="B46" s="14" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>AI-fill / AI draft</t>
         </is>
       </c>
-      <c r="C46" s="15" t="inlineStr">
+      <c r="C47" s="15" t="inlineStr">
         <is>
           <t>Any canvas</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>Click AI-fill / AI draft.</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>It says “queued — coming soon”.</t>
         </is>
       </c>
-      <c r="F46" s="16" t="inlineStr">
+      <c r="F47" s="16" t="inlineStr">
         <is>
           <t>It never actually finishes yet — expected, not a bug.</t>
         </is>
       </c>
-      <c r="G46" s="25" t="inlineStr">
+      <c r="G47" s="25" t="inlineStr">
         <is>
           <t>⛔  Not ready (expected)</t>
         </is>
       </c>
-      <c r="H46" s="18" t="inlineStr"/>
-      <c r="I46" s="15" t="inlineStr"/>
-    </row>
-    <row r="47" ht="92" customHeight="1">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="H47" s="18" t="inlineStr"/>
+      <c r="I47" s="15" t="inlineStr"/>
+    </row>
+    <row r="48" ht="92" customHeight="1">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>5.8</t>
         </is>
       </c>
-      <c r="B47" s="20" t="inlineStr">
+      <c r="B48" s="20" t="inlineStr">
         <is>
           <t>Edit &amp; reorder canvas notes</t>
         </is>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C48" s="21" t="inlineStr">
         <is>
           <t>Business Model / Value Proposition / SWOT</t>
         </is>
       </c>
-      <c r="D47" s="21" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>Click a note to edit it in place (Enter saves, Esc cancels). Then hover a note, grab its drag handle, and drag it to reorder within the same box.</t>
         </is>
       </c>
-      <c r="E47" s="21" t="inlineStr">
+      <c r="E48" s="21" t="inlineStr">
         <is>
           <t>The note updates and saves; the reordered notes save in the new order.</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>Emptying a note and pressing Enter deletes it. Reorder stays within one box. “Mission &amp; Vision” is a text box; “Lean Canvas” doesn’t have these yet.</t>
         </is>
       </c>
-      <c r="G47" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H47" s="23" t="inlineStr"/>
-      <c r="I47" s="21" t="inlineStr"/>
-    </row>
-    <row r="48" ht="92" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="G48" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H48" s="23" t="inlineStr"/>
+      <c r="I48" s="21" t="inlineStr"/>
+    </row>
+    <row r="49" ht="92" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>5.9</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>AI budget guardrail</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>Any canvas (AI draft) + the AI usage display</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>Look at the AI-draft buttons and the AI usage display.</t>
         </is>
       </c>
-      <c r="E48" s="15" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
         <is>
           <t>When the workspace is over its daily AI budget, AI-draft buttons show “AI draft paused (until …)” instead of running; the usage display shows tokens used, or “Unlimited” when there’s no cap.</t>
         </is>
       </c>
-      <c r="F48" s="16" t="inlineStr">
+      <c r="F49" s="16" t="inlineStr">
         <is>
           <t>Honest pause — it never pretends to produce an AI result it can’t.</t>
         </is>
       </c>
-      <c r="G48" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H48" s="18" t="inlineStr"/>
-      <c r="I48" s="15" t="inlineStr"/>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+      <c r="G49" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H49" s="18" t="inlineStr"/>
+      <c r="I49" s="15" t="inlineStr"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="12" t="inlineStr">
         <is>
           <t>6 · Notifications, Journal &amp; Learning</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="92" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
+    <row r="51" ht="92" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>Notifications inbox</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>Bell / Notifications</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>Open it, mark one read, and “mark all read”.</t>
         </is>
       </c>
-      <c r="E50" s="15" t="inlineStr">
+      <c r="E51" s="15" t="inlineStr">
         <is>
           <t>The unread count updates.</t>
         </is>
       </c>
-      <c r="F50" s="16" t="inlineStr">
+      <c r="F51" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G50" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H50" s="18" t="inlineStr"/>
-      <c r="I50" s="15" t="inlineStr"/>
-    </row>
-    <row r="51" ht="92" customHeight="1">
-      <c r="A51" s="19" t="inlineStr">
+      <c r="G51" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H51" s="18" t="inlineStr"/>
+      <c r="I51" s="15" t="inlineStr"/>
+    </row>
+    <row r="52" ht="92" customHeight="1">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B51" s="20" t="inlineStr">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>Email preferences</t>
         </is>
       </c>
-      <c r="C51" s="21" t="inlineStr">
+      <c r="C52" s="21" t="inlineStr">
         <is>
           <t>Notifications → Preferences</t>
         </is>
       </c>
-      <c r="D51" s="21" t="inlineStr">
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>Toggle the master email switch and the 5 category switches.</t>
         </is>
       </c>
-      <c r="E51" s="21" t="inlineStr">
+      <c r="E52" s="21" t="inlineStr">
         <is>
           <t>They save.</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>The “Digest &amp; quiet hours” and “Announcements” tabs are demo-only for now.</t>
         </is>
       </c>
-      <c r="G51" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H51" s="23" t="inlineStr"/>
-      <c r="I51" s="21" t="inlineStr"/>
-    </row>
-    <row r="52" ht="92" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H52" s="23" t="inlineStr"/>
+      <c r="I52" s="21" t="inlineStr"/>
+    </row>
+    <row r="53" ht="92" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="B52" s="14" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>Read the journal</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="C53" s="15" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>Read journal entries.</t>
         </is>
       </c>
-      <c r="E52" s="15" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
         <is>
           <t>Reading works.</t>
         </is>
       </c>
-      <c r="F52" s="16" t="inlineStr">
+      <c r="F53" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G52" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H52" s="18" t="inlineStr"/>
-      <c r="I52" s="15" t="inlineStr"/>
-    </row>
-    <row r="53" ht="92" customHeight="1">
-      <c r="A53" s="19" t="inlineStr">
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr"/>
+      <c r="I53" s="15" t="inlineStr"/>
+    </row>
+    <row r="54" ht="92" customHeight="1">
+      <c r="A54" s="19" t="inlineStr">
         <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="B53" s="20" t="inlineStr">
+      <c r="B54" s="20" t="inlineStr">
         <is>
           <t>Save a new journal entry</t>
         </is>
       </c>
-      <c r="C53" s="21" t="inlineStr">
+      <c r="C54" s="21" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="D53" s="21" t="inlineStr">
+      <c r="D54" s="21" t="inlineStr">
         <is>
           <t>Try to save a new entry.</t>
         </is>
       </c>
-      <c r="E53" s="21" t="inlineStr">
+      <c r="E54" s="21" t="inlineStr">
         <is>
           <t>It fails gracefully — it doesn’t crash the page.</t>
         </is>
       </c>
-      <c r="F53" s="22" t="inlineStr">
+      <c r="F54" s="22" t="inlineStr">
         <is>
           <t>Saving isn’t set up on the test server yet — expected to fail softly.</t>
         </is>
       </c>
-      <c r="G53" s="25" t="inlineStr">
+      <c r="G54" s="25" t="inlineStr">
         <is>
           <t>⛔  Not ready (expected)</t>
         </is>
       </c>
-      <c r="H53" s="23" t="inlineStr"/>
-      <c r="I53" s="21" t="inlineStr"/>
-    </row>
-    <row r="54" ht="92" customHeight="1">
-      <c r="A54" s="13" t="inlineStr">
+      <c r="H54" s="23" t="inlineStr"/>
+      <c r="I54" s="21" t="inlineStr"/>
+    </row>
+    <row r="55" ht="92" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
         <is>
           <t>6.5</t>
         </is>
       </c>
-      <c r="B54" s="14" t="inlineStr">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>Learning academy</t>
         </is>
       </c>
-      <c r="C54" s="15" t="inlineStr">
+      <c r="C55" s="15" t="inlineStr">
         <is>
           <t>Academy</t>
         </is>
       </c>
-      <c r="D54" s="15" t="inlineStr">
+      <c r="D55" s="15" t="inlineStr">
         <is>
           <t>Browse courses / articles / paths / certificates, enroll, and complete a lesson.</t>
         </is>
       </c>
-      <c r="E54" s="15" t="inlineStr">
+      <c r="E55" s="15" t="inlineStr">
         <is>
           <t>These work and save.</t>
         </is>
       </c>
-      <c r="F54" s="16" t="inlineStr">
+      <c r="F55" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G54" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H54" s="18" t="inlineStr"/>
-      <c r="I54" s="15" t="inlineStr"/>
-    </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr"/>
+      <c r="I55" s="15" t="inlineStr"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="12" t="inlineStr">
         <is>
           <t>7 · Documents</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="92" customHeight="1">
-      <c r="A56" s="13" t="inlineStr">
+    <row r="57" ht="92" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>Files</t>
         </is>
       </c>
-      <c r="C56" s="15" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>Upload, list, and delete a file.</t>
         </is>
       </c>
-      <c r="E56" s="15" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>All three work.</t>
         </is>
       </c>
-      <c r="F56" s="16" t="inlineStr">
+      <c r="F57" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G56" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H56" s="18" t="inlineStr"/>
-      <c r="I56" s="15" t="inlineStr"/>
-    </row>
-    <row r="57" ht="92" customHeight="1">
-      <c r="A57" s="19" t="inlineStr">
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr"/>
+      <c r="I57" s="15" t="inlineStr"/>
+    </row>
+    <row r="58" ht="92" customHeight="1">
+      <c r="A58" s="19" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="B57" s="20" t="inlineStr">
+      <c r="B58" s="20" t="inlineStr">
         <is>
           <t>Share a document</t>
         </is>
       </c>
-      <c r="C57" s="21" t="inlineStr">
+      <c r="C58" s="21" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="D57" s="21" t="inlineStr">
+      <c r="D58" s="21" t="inlineStr">
         <is>
           <t>Share a document, then remove the share.</t>
         </is>
       </c>
-      <c r="E57" s="21" t="inlineStr">
+      <c r="E58" s="21" t="inlineStr">
         <is>
           <t>The share list updates.</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G57" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H57" s="23" t="inlineStr"/>
-      <c r="I57" s="21" t="inlineStr"/>
-    </row>
-    <row r="58" ht="92" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="G58" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H58" s="23" t="inlineStr"/>
+      <c r="I58" s="21" t="inlineStr"/>
+    </row>
+    <row r="59" ht="92" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="B58" s="14" t="inlineStr">
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>Signature requests</t>
         </is>
       </c>
-      <c r="C58" s="15" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
         <is>
           <t>Documents → Signatures</t>
         </is>
       </c>
-      <c r="D58" s="15" t="inlineStr">
+      <c r="D59" s="15" t="inlineStr">
         <is>
           <t>Send, remind, or cancel a signature request.</t>
         </is>
       </c>
-      <c r="E58" s="15" t="inlineStr">
+      <c r="E59" s="15" t="inlineStr">
         <is>
           <t>The status reflects what you did.</t>
         </is>
       </c>
-      <c r="F58" s="16" t="inlineStr">
+      <c r="F59" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G58" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H58" s="18" t="inlineStr"/>
-      <c r="I58" s="15" t="inlineStr"/>
-    </row>
-    <row r="59" ht="92" customHeight="1">
-      <c r="A59" s="19" t="inlineStr">
+      <c r="G59" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr"/>
+      <c r="I59" s="15" t="inlineStr"/>
+    </row>
+    <row r="60" ht="92" customHeight="1">
+      <c r="A60" s="19" t="inlineStr">
         <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="B59" s="20" t="inlineStr">
+      <c r="B60" s="20" t="inlineStr">
         <is>
           <t>Create from a template</t>
         </is>
       </c>
-      <c r="C59" s="21" t="inlineStr">
+      <c r="C60" s="21" t="inlineStr">
         <is>
           <t>Documents → Templates</t>
         </is>
       </c>
-      <c r="D59" s="21" t="inlineStr">
+      <c r="D60" s="21" t="inlineStr">
         <is>
           <t>Create a document from a template.</t>
         </is>
       </c>
-      <c r="E59" s="21" t="inlineStr">
+      <c r="E60" s="21" t="inlineStr">
         <is>
           <t>It creates the document.</t>
         </is>
       </c>
-      <c r="F59" s="22" t="inlineStr">
+      <c r="F60" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G59" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H59" s="23" t="inlineStr"/>
-      <c r="I59" s="21" t="inlineStr"/>
-    </row>
-    <row r="60" ht="92" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="G60" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H60" s="23" t="inlineStr"/>
+      <c r="I60" s="21" t="inlineStr"/>
+    </row>
+    <row r="61" ht="92" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
         <is>
           <t>7.5</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>Edit &amp; save a document</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
+      <c r="C61" s="15" t="inlineStr">
         <is>
           <t>Documents → open a document</t>
         </is>
       </c>
-      <c r="D60" s="15" t="inlineStr">
+      <c r="D61" s="15" t="inlineStr">
         <is>
           <t>Open the editor, make edits, and save.</t>
         </is>
       </c>
-      <c r="E60" s="15" t="inlineStr">
+      <c r="E61" s="15" t="inlineStr">
         <is>
           <t>Your edits save.</t>
         </is>
       </c>
-      <c r="F60" s="16" t="inlineStr">
+      <c r="F61" s="16" t="inlineStr">
         <is>
           <t>Documents don’t auto-save — click Save. If it was changed elsewhere you get a “reload” banner and it won’t overwrite.</t>
         </is>
       </c>
-      <c r="G60" s="24" t="inlineStr">
+      <c r="G61" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H60" s="18" t="inlineStr"/>
-      <c r="I60" s="15" t="inlineStr"/>
-    </row>
-    <row r="61" ht="92" customHeight="1">
-      <c r="A61" s="19" t="inlineStr">
+      <c r="H61" s="18" t="inlineStr"/>
+      <c r="I61" s="15" t="inlineStr"/>
+    </row>
+    <row r="62" ht="92" customHeight="1">
+      <c r="A62" s="19" t="inlineStr">
         <is>
           <t>7.6</t>
         </is>
       </c>
-      <c r="B61" s="20" t="inlineStr">
+      <c r="B62" s="20" t="inlineStr">
         <is>
           <t>Open a real emailed sign/share link</t>
         </is>
       </c>
-      <c r="C61" s="21" t="inlineStr">
+      <c r="C62" s="21" t="inlineStr">
         <is>
           <t>The sign/share link</t>
         </is>
       </c>
-      <c r="D61" s="21" t="inlineStr">
+      <c r="D62" s="21" t="inlineStr">
         <is>
           <t>Open a real emailed link.</t>
         </is>
       </c>
-      <c r="E61" s="21" t="inlineStr">
+      <c r="E62" s="21" t="inlineStr">
         <is>
           <t>The recipient page works when opened on the app website.</t>
         </is>
       </c>
-      <c r="F61" s="22" t="inlineStr">
+      <c r="F62" s="22" t="inlineStr">
         <is>
           <t>Straight from an email it may show a raw data page — open it on the app website instead.</t>
         </is>
       </c>
-      <c r="G61" s="25" t="inlineStr">
+      <c r="G62" s="25" t="inlineStr">
         <is>
           <t>⛔  Not ready (expected)</t>
         </is>
       </c>
-      <c r="H61" s="23" t="inlineStr"/>
-      <c r="I61" s="21" t="inlineStr"/>
-    </row>
-    <row r="62" ht="92" customHeight="1">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="H62" s="23" t="inlineStr"/>
+      <c r="I62" s="21" t="inlineStr"/>
+    </row>
+    <row r="63" ht="92" customHeight="1">
+      <c r="A63" s="13" t="inlineStr">
         <is>
           <t>7.7</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>Edit a document’s sections</t>
         </is>
       </c>
-      <c r="C62" s="15" t="inlineStr">
+      <c r="C63" s="15" t="inlineStr">
         <is>
           <t>Documents → open a document</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
+      <c r="D63" s="15" t="inlineStr">
         <is>
           <t>Add a section, delete one, drag a section to reorder (or use the up/down arrows), and rename a heading. Then Save.</t>
         </is>
       </c>
-      <c r="E62" s="15" t="inlineStr">
+      <c r="E63" s="15" t="inlineStr">
         <is>
           <t>All the section changes save after you click Save.</t>
         </is>
       </c>
-      <c r="F62" s="16" t="inlineStr">
+      <c r="F63" s="16" t="inlineStr">
         <is>
           <t>Documents don’t auto-save — you must click Save. Headings used to be read-only.</t>
         </is>
       </c>
-      <c r="G62" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H62" s="18" t="inlineStr"/>
-      <c r="I62" s="15" t="inlineStr"/>
-    </row>
-    <row r="63" ht="92" customHeight="1">
-      <c r="A63" s="19" t="inlineStr">
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr"/>
+      <c r="I63" s="15" t="inlineStr"/>
+    </row>
+    <row r="64" ht="92" customHeight="1">
+      <c r="A64" s="19" t="inlineStr">
         <is>
           <t>7.8</t>
         </is>
       </c>
-      <c r="B63" s="20" t="inlineStr">
+      <c r="B64" s="20" t="inlineStr">
         <is>
           <t>Sign a document</t>
         </is>
       </c>
-      <c r="C63" s="21" t="inlineStr">
+      <c r="C64" s="21" t="inlineStr">
         <is>
           <t>The signing link, on the app website</t>
         </is>
       </c>
-      <c r="D63" s="21" t="inlineStr">
+      <c r="D64" s="21" t="inlineStr">
         <is>
           <t>Read the preview, type your full name (shown styled like a signature), tick the “I agree…” box, then Sign.</t>
         </is>
       </c>
-      <c r="E63" s="21" t="inlineStr">
+      <c r="E64" s="21" t="inlineStr">
         <is>
           <t>Your typed name is accepted and you see a “signed — thank you” confirmation.</t>
         </is>
       </c>
-      <c r="F63" s="22" t="inlineStr">
+      <c r="F64" s="22" t="inlineStr">
         <is>
           <t>It’s a typed signature (no drawing pad). The Sign button stays disabled until you tick consent.</t>
         </is>
       </c>
-      <c r="G63" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H63" s="23" t="inlineStr"/>
-      <c r="I63" s="21" t="inlineStr"/>
+      <c r="G64" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H64" s="23" t="inlineStr"/>
+      <c r="I64" s="21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A49:I49"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A32:I32"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A56:I56"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A39:I39"/>
-    <mergeCell ref="A55:I55"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A26:I26"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
+    <dataValidation sqref="H4:H64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Make AI Co-Founder chat honest (no fabricated replies)
The conversational AI Co-Founder has no backend (the BE's own
fe-integration-guide-ai-cofounder.md confirms the /ai router exposes
only GET /ai/status, no conversation endpoint). The FE faked it with two
seeded fake conversations (invented runway/finance data) and a hardcoded
typewriter reply plus fake sources/reasoning/action chips.

- useAICoFounder: drop the fake seed conversations; sendMessage now returns
  one honest 'not connected yet' reply with no fabricated reasoning/sources/
  chips; stamp new conversations with an ISO lastMessageAt (fixes 'Invalid
  Date' in the list)
- /ai page + ai-drawer: honest 'coming soon' empty state that points to where
  the AI actually works (dashboard briefing, mission reasons, health tips)
- Log the chat backend as a BE follow-up (backend-requests-ui-gaps §7)
- Docs: SOP module-38, frontend checklist, QA checklist + xlsx (case 1.19)
</commit_message>
<xml_diff>
--- a/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
+++ b/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
@@ -882,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1659,1621 +1659,1660 @@
       <c r="H21" s="23" t="inlineStr"/>
       <c r="I21" s="21" t="inlineStr"/>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="22" ht="92" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>1.19</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>AI Co-Founder chat</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>AI Co-Founder page and the floating chat button</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Open it, type a question (e.g. “How long is my runway?”) and press Send.</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>A “Coming soon” message, and an honest reply that the AI Co-Founder isn’t connected yet.</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>It must NOT make up an answer (no invented numbers, sources or buttons) — the chat has no backend yet. The real AI shows up in your dashboard briefing, today’s mission reasons and health tips.</t>
+        </is>
+      </c>
+      <c r="G22" s="25" t="inlineStr">
+        <is>
+          <t>⛔  Not ready (expected)</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr"/>
+      <c r="I22" s="15" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>2 · Health score</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="92" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+    <row r="24" ht="92" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Overview loads</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Open Health.</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>You see your overall score and the five areas.</t>
         </is>
       </c>
-      <c r="F23" s="16" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>A thriving account shows around 90.</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H23" s="18" t="inlineStr"/>
-      <c r="I23" s="15" t="inlineStr"/>
-    </row>
-    <row r="24" ht="92" customHeight="1">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr"/>
+      <c r="I24" s="15" t="inlineStr"/>
+    </row>
+    <row r="25" ht="92" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>Open the Financial area</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>Health → Dimensions → Financial</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Open the “Financial” area.</t>
         </is>
       </c>
-      <c r="E24" s="21" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>It loads with its details.</t>
         </is>
       </c>
-      <c r="F24" s="22" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>Make sure “Financial” isn’t blank (it’s stored under a different name internally).</t>
         </is>
       </c>
-      <c r="G24" s="24" t="inlineStr">
+      <c r="G25" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H24" s="23" t="inlineStr"/>
-      <c r="I24" s="21" t="inlineStr"/>
-    </row>
-    <row r="25" ht="92" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="H25" s="23" t="inlineStr"/>
+      <c r="I25" s="21" t="inlineStr"/>
+    </row>
+    <row r="26" ht="92" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Change the history range</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Health → Trend history</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Switch the time range (7d / 30d / 90d / all).</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>The chart updates to match the range you picked.</t>
         </is>
       </c>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H25" s="18" t="inlineStr"/>
-      <c r="I25" s="15" t="inlineStr"/>
-    </row>
-    <row r="26" ht="92" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr"/>
+      <c r="I26" s="15" t="inlineStr"/>
+    </row>
+    <row r="27" ht="92" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>Benchmarks</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C27" s="21" t="inlineStr">
         <is>
           <t>Health → Benchmarks</t>
         </is>
       </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>Open Benchmarks.</t>
         </is>
       </c>
-      <c r="E26" s="21" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>You see comparison data, OR an honest “not enough data yet” message.</t>
         </is>
       </c>
-      <c r="F26" s="22" t="inlineStr">
+      <c r="F27" s="22" t="inlineStr">
         <is>
           <t>If empty it should SAY so — not show made-up numbers.</t>
         </is>
       </c>
-      <c r="G26" s="24" t="inlineStr">
+      <c r="G27" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H26" s="23" t="inlineStr"/>
-      <c r="I26" s="21" t="inlineStr"/>
-    </row>
-    <row r="27" ht="92" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="H27" s="23" t="inlineStr"/>
+      <c r="I27" s="21" t="inlineStr"/>
+    </row>
+    <row r="28" ht="92" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Accept / dismiss a recommendation</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>Health → Recommendations</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>Accept or dismiss a recommendation.</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>It resolves and leaves the list.</t>
         </is>
       </c>
-      <c r="F27" s="16" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>The main test account may have zero — try a lower-scoring account. Acting on the same one twice may say “already resolved”.</t>
         </is>
       </c>
-      <c r="G27" s="24" t="inlineStr">
+      <c r="G28" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H27" s="18" t="inlineStr"/>
-      <c r="I27" s="15" t="inlineStr"/>
-    </row>
-    <row r="28" ht="92" customHeight="1">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="H28" s="18" t="inlineStr"/>
+      <c r="I28" s="15" t="inlineStr"/>
+    </row>
+    <row r="29" ht="92" customHeight="1">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Charts show real data</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>Health → overview, Trend history, a single dimension</t>
         </is>
       </c>
-      <c r="D28" s="21" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>Look at the three charts: the “Dimension balance” wheel, the “Score over time” chart, and a dimension’s trend chart.</t>
         </is>
       </c>
-      <c r="E28" s="21" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>The wheel shows your five scores; the score-over-time chart has a 0–100 scale and a tooltip; a dimension shows its own trend.</t>
         </is>
       </c>
-      <c r="F28" s="22" t="inlineStr">
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>Only one assessment done → the score chart shows a single dot (correct). The dashboard KPI cards no longer show a mini trend line (there’s no real trend data for them).</t>
         </is>
       </c>
-      <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H28" s="23" t="inlineStr"/>
-      <c r="I28" s="21" t="inlineStr"/>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr"/>
+      <c r="I29" s="21" t="inlineStr"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>3 · Today’s Mission</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="92" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
+    <row r="31" ht="92" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>Load today’s mission</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>Today’s Mission</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>You see today’s tasks and your streak.</t>
         </is>
       </c>
-      <c r="F30" s="16" t="inlineStr">
+      <c r="F31" s="16" t="inlineStr">
         <is>
           <t>A weekend-off day can legitimately have no tasks.</t>
         </is>
       </c>
-      <c r="G30" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H30" s="18" t="inlineStr"/>
-      <c r="I30" s="15" t="inlineStr"/>
-    </row>
-    <row r="31" ht="92" customHeight="1">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H31" s="18" t="inlineStr"/>
+      <c r="I31" s="15" t="inlineStr"/>
+    </row>
+    <row r="32" ht="92" customHeight="1">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>Task actions</t>
         </is>
       </c>
-      <c r="C31" s="21" t="inlineStr">
+      <c r="C32" s="21" t="inlineStr">
         <is>
           <t>Today’s Mission</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
         <is>
           <t>Complete, snooze, reject, add, or reorder a task.</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
+      <c r="E32" s="21" t="inlineStr">
         <is>
           <t>Each updates, and the list and streak refresh correctly.</t>
         </is>
       </c>
-      <c r="F31" s="22" t="inlineStr">
+      <c r="F32" s="22" t="inlineStr">
         <is>
           <t>Completing a task is final — you can’t un-complete it.</t>
         </is>
       </c>
-      <c r="G31" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H31" s="23" t="inlineStr"/>
-      <c r="I31" s="21" t="inlineStr"/>
-    </row>
-    <row r="32" ht="92" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H32" s="23" t="inlineStr"/>
+      <c r="I32" s="21" t="inlineStr"/>
+    </row>
+    <row r="33" ht="92" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Reject a task</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>Today’s Mission</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>Reject a task and pick a reason.</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>It’s rejected with the reason you chose.</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="F33" s="16" t="inlineStr">
         <is>
           <t>Use the reason chips provided (don’t type your own).</t>
         </is>
       </c>
-      <c r="G32" s="24" t="inlineStr">
+      <c r="G33" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H32" s="18" t="inlineStr"/>
-      <c r="I32" s="15" t="inlineStr"/>
-    </row>
-    <row r="33" ht="92" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="H33" s="18" t="inlineStr"/>
+      <c r="I33" s="15" t="inlineStr"/>
+    </row>
+    <row r="34" ht="92" customHeight="1">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>Mission settings</t>
         </is>
       </c>
-      <c r="C33" s="21" t="inlineStr">
+      <c r="C34" s="21" t="inlineStr">
         <is>
           <t>Mission → Settings</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>Change mission size, delivery time, or the weekends option.</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>Your settings save.</t>
         </is>
       </c>
-      <c r="F33" s="22" t="inlineStr">
+      <c r="F34" s="22" t="inlineStr">
         <is>
           <t>Time flips between 12-hour and 24-hour; “weekends off” is the opposite of “weekend missions”.</t>
         </is>
       </c>
-      <c r="G33" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H33" s="23" t="inlineStr"/>
-      <c r="I33" s="21" t="inlineStr"/>
-    </row>
-    <row r="34" ht="92" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H34" s="23" t="inlineStr"/>
+      <c r="I34" s="21" t="inlineStr"/>
+    </row>
+    <row r="35" ht="92" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>History pages</t>
         </is>
       </c>
-      <c r="C34" s="15" t="inlineStr">
+      <c r="C35" s="15" t="inlineStr">
         <is>
           <t>Mission → Completed / Streaks / Upcoming</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>Open each.</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="E35" s="15" t="inlineStr">
         <is>
           <t>They fill with your real history.</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>No history yet → an honest empty message.</t>
         </is>
       </c>
-      <c r="G34" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H34" s="18" t="inlineStr"/>
-      <c r="I34" s="15" t="inlineStr"/>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H35" s="18" t="inlineStr"/>
+      <c r="I35" s="15" t="inlineStr"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>4 · Roadmap</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="92" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
+    <row r="37" ht="92" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>Load the roadmap</t>
         </is>
       </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
         <is>
           <t>Roadmap</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="E37" s="15" t="inlineStr">
         <is>
           <t>You see phases → milestones → tasks.</t>
         </is>
       </c>
-      <c r="F36" s="16" t="inlineStr">
+      <c r="F37" s="16" t="inlineStr">
         <is>
           <t>A “slipped / behind” count shows if any dates have slipped.</t>
         </is>
       </c>
-      <c r="G36" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H36" s="18" t="inlineStr"/>
-      <c r="I36" s="15" t="inlineStr"/>
-    </row>
-    <row r="37" ht="92" customHeight="1">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H37" s="18" t="inlineStr"/>
+      <c r="I37" s="15" t="inlineStr"/>
+    </row>
+    <row r="38" ht="92" customHeight="1">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>Add / edit / delete</t>
         </is>
       </c>
-      <c r="C37" s="21" t="inlineStr">
+      <c r="C38" s="21" t="inlineStr">
         <is>
           <t>Roadmap</t>
         </is>
       </c>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>Add, edit, or delete a phase, milestone or task.</t>
         </is>
       </c>
-      <c r="E37" s="21" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>The change saves and the roadmap updates.</t>
         </is>
       </c>
-      <c r="F37" s="22" t="inlineStr">
+      <c r="F38" s="22" t="inlineStr">
         <is>
           <t>Editors only — a mentor/viewer can’t make changes.</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H37" s="23" t="inlineStr"/>
-      <c r="I37" s="21" t="inlineStr"/>
-    </row>
-    <row r="38" ht="92" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H38" s="23" t="inlineStr"/>
+      <c r="I38" s="21" t="inlineStr"/>
+    </row>
+    <row r="39" ht="92" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>Block a dependency loop</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Dependencies</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>Try to link two tasks so they depend on each other in a circle.</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
+      <c r="E39" s="15" t="inlineStr">
         <is>
           <t>The app refuses to create the circular link.</t>
         </is>
       </c>
-      <c r="F38" s="16" t="inlineStr">
+      <c r="F39" s="16" t="inlineStr">
         <is>
           <t>It should block the loop.</t>
         </is>
       </c>
-      <c r="G38" s="24" t="inlineStr">
+      <c r="G39" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H38" s="18" t="inlineStr"/>
-      <c r="I38" s="15" t="inlineStr"/>
-    </row>
-    <row r="39" ht="92" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
+      <c r="H39" s="18" t="inlineStr"/>
+      <c r="I39" s="15" t="inlineStr"/>
+    </row>
+    <row r="40" ht="92" customHeight="1">
+      <c r="A40" s="19" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="B39" s="20" t="inlineStr">
+      <c r="B40" s="20" t="inlineStr">
         <is>
           <t>Apply a template</t>
         </is>
       </c>
-      <c r="C39" s="21" t="inlineStr">
+      <c r="C40" s="21" t="inlineStr">
         <is>
           <t>Roadmap → Templates</t>
         </is>
       </c>
-      <c r="D39" s="21" t="inlineStr">
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>Browse the gallery and apply a template.</t>
         </is>
       </c>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="E40" s="21" t="inlineStr">
         <is>
           <t>The roadmap updates from the template.</t>
         </is>
       </c>
-      <c r="F39" s="22" t="inlineStr">
+      <c r="F40" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G39" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H39" s="23" t="inlineStr"/>
-      <c r="I39" s="21" t="inlineStr"/>
-    </row>
-    <row r="40" ht="92" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr"/>
+      <c r="I40" s="21" t="inlineStr"/>
+    </row>
+    <row r="41" ht="92" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>AI Re-plan — preview &amp; apply</t>
         </is>
       </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Re-Plan</t>
         </is>
       </c>
-      <c r="D40" s="15" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>Preview an AI re-plan, then apply it, and check history.</t>
         </is>
       </c>
-      <c r="E40" s="15" t="inlineStr">
+      <c r="E41" s="15" t="inlineStr">
         <is>
           <t>Preview shows changes; applying updates the plan; history logs it.</t>
         </is>
       </c>
-      <c r="F40" s="16" t="inlineStr">
+      <c r="F41" s="16" t="inlineStr">
         <is>
           <t>Nothing changes until you click Apply.</t>
         </is>
       </c>
-      <c r="G40" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H40" s="18" t="inlineStr"/>
-      <c r="I40" s="15" t="inlineStr"/>
-    </row>
-    <row r="41" ht="92" customHeight="1">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H41" s="18" t="inlineStr"/>
+      <c r="I41" s="15" t="inlineStr"/>
+    </row>
+    <row r="42" ht="92" customHeight="1">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
       </c>
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>Move a task on the Kanban board</t>
         </is>
       </c>
-      <c r="C41" s="21" t="inlineStr">
+      <c r="C42" s="21" t="inlineStr">
         <is>
           <t>Roadmap → Kanban (Status view)</t>
         </is>
       </c>
-      <c r="D41" s="21" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>Drag a task card between columns (To Do / In Progress / Done).</t>
         </is>
       </c>
-      <c r="E41" s="21" t="inlineStr">
+      <c r="E42" s="21" t="inlineStr">
         <is>
           <t>The card moves and the change stays after a refresh.</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F42" s="22" t="inlineStr">
         <is>
           <t>Mentor/viewer → the card snaps back (permission working). The “Phase” view isn’t drag-and-drop; tap a card to open it.</t>
         </is>
       </c>
-      <c r="G41" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H41" s="23" t="inlineStr"/>
-      <c r="I41" s="21" t="inlineStr"/>
-    </row>
-    <row r="42" ht="92" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H42" s="23" t="inlineStr"/>
+      <c r="I42" s="21" t="inlineStr"/>
+    </row>
+    <row r="43" ht="92" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Re-plan — date changes &amp; history</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>Roadmap → Re-Plan</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>Generate a re-plan; expand a past entry under “Re-plan History”.</t>
         </is>
       </c>
-      <c r="E42" s="15" t="inlineStr">
+      <c r="E43" s="15" t="inlineStr">
         <is>
           <t>Each change shows old date → new date and how far it moved (e.g. “+17 days”); history entries expand to their before/after dates.</t>
         </is>
       </c>
-      <c r="F42" s="16" t="inlineStr">
+      <c r="F43" s="16" t="inlineStr">
         <is>
           <t>Deltas come from the real dates — nothing invented.</t>
         </is>
       </c>
-      <c r="G42" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H42" s="18" t="inlineStr"/>
-      <c r="I42" s="15" t="inlineStr"/>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H43" s="18" t="inlineStr"/>
+      <c r="I43" s="15" t="inlineStr"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>5 · Business Builder</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="92" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
+    <row r="45" ht="92" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>Overview</t>
         </is>
       </c>
-      <c r="C44" s="15" t="inlineStr">
+      <c r="C45" s="15" t="inlineStr">
         <is>
           <t>Business Builder</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D45" s="15" t="inlineStr">
         <is>
           <t>Open it.</t>
         </is>
       </c>
-      <c r="E44" s="15" t="inlineStr">
+      <c r="E45" s="15" t="inlineStr">
         <is>
           <t>You see each canvas with a completion %.</t>
         </is>
       </c>
-      <c r="F44" s="16" t="inlineStr">
+      <c r="F45" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G44" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H44" s="18" t="inlineStr"/>
-      <c r="I44" s="15" t="inlineStr"/>
-    </row>
-    <row r="45" ht="92" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H45" s="18" t="inlineStr"/>
+      <c r="I45" s="15" t="inlineStr"/>
+    </row>
+    <row r="46" ht="92" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B46" s="20" t="inlineStr">
         <is>
           <t>Lean canvas saves</t>
         </is>
       </c>
-      <c r="C45" s="21" t="inlineStr">
+      <c r="C46" s="21" t="inlineStr">
         <is>
           <t>Business Builder → Lean Canvas</t>
         </is>
       </c>
-      <c r="D45" s="21" t="inlineStr">
+      <c r="D46" s="21" t="inlineStr">
         <is>
           <t>Edit some blocks and wait a moment.</t>
         </is>
       </c>
-      <c r="E45" s="21" t="inlineStr">
+      <c r="E46" s="21" t="inlineStr">
         <is>
           <t>It saves on its own.</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F46" s="22" t="inlineStr">
         <is>
           <t>Advanced: editing the same canvas in two tabs may briefly show it reconciling — that’s the safety check.</t>
         </is>
       </c>
-      <c r="G45" s="24" t="inlineStr">
+      <c r="G46" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H45" s="23" t="inlineStr"/>
-      <c r="I45" s="21" t="inlineStr"/>
-    </row>
-    <row r="46" ht="92" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="H46" s="23" t="inlineStr"/>
+      <c r="I46" s="21" t="inlineStr"/>
+    </row>
+    <row r="47" ht="92" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="B46" s="14" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>Canvases save automatically</t>
         </is>
       </c>
-      <c r="C46" s="15" t="inlineStr">
+      <c r="C47" s="15" t="inlineStr">
         <is>
           <t>Business Model / Value Proposition / SWOT / Mission &amp; Vision</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>Edit and pause.</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>It saves on its own after you stop typing.</t>
         </is>
       </c>
-      <c r="F46" s="16" t="inlineStr">
+      <c r="F47" s="16" t="inlineStr">
         <is>
           <t>Pause after typing to let it save.</t>
         </is>
       </c>
-      <c r="G46" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H46" s="18" t="inlineStr"/>
-      <c r="I46" s="15" t="inlineStr"/>
-    </row>
-    <row r="47" ht="92" customHeight="1">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H47" s="18" t="inlineStr"/>
+      <c r="I47" s="15" t="inlineStr"/>
+    </row>
+    <row r="48" ht="92" customHeight="1">
+      <c r="A48" s="19" t="inlineStr">
         <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="B47" s="20" t="inlineStr">
+      <c r="B48" s="20" t="inlineStr">
         <is>
           <t>Records — add / edit / delete</t>
         </is>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C48" s="21" t="inlineStr">
         <is>
           <t>Personas / Competitive / Pricing / Revenue</t>
         </is>
       </c>
-      <c r="D47" s="21" t="inlineStr">
+      <c r="D48" s="21" t="inlineStr">
         <is>
           <t>Create, edit, and delete a record.</t>
         </is>
       </c>
-      <c r="E47" s="21" t="inlineStr">
+      <c r="E48" s="21" t="inlineStr">
         <is>
           <t>The list updates.</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>Leaving a required field empty shows a validation message. Pricing has tiers inside it.</t>
         </is>
       </c>
-      <c r="G47" s="24" t="inlineStr">
+      <c r="G48" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H47" s="23" t="inlineStr"/>
-      <c r="I47" s="21" t="inlineStr"/>
-    </row>
-    <row r="48" ht="92" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="H48" s="23" t="inlineStr"/>
+      <c r="I48" s="21" t="inlineStr"/>
+    </row>
+    <row r="49" ht="92" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>Suggestions</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>Business Builder → Suggestions</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>Approve or reject a suggestion.</t>
         </is>
       </c>
-      <c r="E48" s="15" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
         <is>
           <t>It applies or updates.</t>
         </is>
       </c>
-      <c r="F48" s="16" t="inlineStr">
+      <c r="F49" s="16" t="inlineStr">
         <is>
           <t>May say “no longer pending” if the canvas has moved on.</t>
         </is>
       </c>
-      <c r="G48" s="24" t="inlineStr">
+      <c r="G49" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H48" s="18" t="inlineStr"/>
-      <c r="I48" s="15" t="inlineStr"/>
-    </row>
-    <row r="49" ht="92" customHeight="1">
-      <c r="A49" s="19" t="inlineStr">
+      <c r="H49" s="18" t="inlineStr"/>
+      <c r="I49" s="15" t="inlineStr"/>
+    </row>
+    <row r="50" ht="92" customHeight="1">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>5.6</t>
         </is>
       </c>
-      <c r="B49" s="20" t="inlineStr">
+      <c r="B50" s="20" t="inlineStr">
         <is>
           <t>Positioning map</t>
         </is>
       </c>
-      <c r="C49" s="21" t="inlineStr">
+      <c r="C50" s="21" t="inlineStr">
         <is>
           <t>Business Builder → Positioning map</t>
         </is>
       </c>
-      <c r="D49" s="21" t="inlineStr">
+      <c r="D50" s="21" t="inlineStr">
         <is>
           <t>Edit the axes.</t>
         </is>
       </c>
-      <c r="E49" s="21" t="inlineStr">
+      <c r="E50" s="21" t="inlineStr">
         <is>
           <t>Competitors plot against your saved axes.</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F50" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G49" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H49" s="23" t="inlineStr"/>
-      <c r="I49" s="21" t="inlineStr"/>
-    </row>
-    <row r="50" ht="92" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="G50" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H50" s="23" t="inlineStr"/>
+      <c r="I50" s="21" t="inlineStr"/>
+    </row>
+    <row r="51" ht="92" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
         <is>
           <t>5.7</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>AI-fill / AI draft</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>Any canvas</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>Click AI-fill / AI draft.</t>
         </is>
       </c>
-      <c r="E50" s="15" t="inlineStr">
+      <c r="E51" s="15" t="inlineStr">
         <is>
           <t>It says “queued — coming soon”.</t>
         </is>
       </c>
-      <c r="F50" s="16" t="inlineStr">
+      <c r="F51" s="16" t="inlineStr">
         <is>
           <t>It never actually finishes yet — expected, not a bug.</t>
         </is>
       </c>
-      <c r="G50" s="25" t="inlineStr">
+      <c r="G51" s="25" t="inlineStr">
         <is>
           <t>⛔  Not ready (expected)</t>
         </is>
       </c>
-      <c r="H50" s="18" t="inlineStr"/>
-      <c r="I50" s="15" t="inlineStr"/>
-    </row>
-    <row r="51" ht="92" customHeight="1">
-      <c r="A51" s="19" t="inlineStr">
+      <c r="H51" s="18" t="inlineStr"/>
+      <c r="I51" s="15" t="inlineStr"/>
+    </row>
+    <row r="52" ht="92" customHeight="1">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>5.8</t>
         </is>
       </c>
-      <c r="B51" s="20" t="inlineStr">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>Edit &amp; reorder canvas notes</t>
         </is>
       </c>
-      <c r="C51" s="21" t="inlineStr">
+      <c r="C52" s="21" t="inlineStr">
         <is>
           <t>Business Model / Value Proposition / SWOT</t>
         </is>
       </c>
-      <c r="D51" s="21" t="inlineStr">
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>Click a note to edit it in place (Enter saves, Esc cancels). Then hover a note, grab its drag handle, and drag it to reorder within the same box.</t>
         </is>
       </c>
-      <c r="E51" s="21" t="inlineStr">
+      <c r="E52" s="21" t="inlineStr">
         <is>
           <t>The note updates and saves; the reordered notes save in the new order.</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>Emptying a note and pressing Enter deletes it. Reorder stays within one box. “Mission &amp; Vision” is a text box; “Lean Canvas” doesn’t have these yet.</t>
         </is>
       </c>
-      <c r="G51" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H51" s="23" t="inlineStr"/>
-      <c r="I51" s="21" t="inlineStr"/>
-    </row>
-    <row r="52" ht="92" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H52" s="23" t="inlineStr"/>
+      <c r="I52" s="21" t="inlineStr"/>
+    </row>
+    <row r="53" ht="92" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>5.9</t>
         </is>
       </c>
-      <c r="B52" s="14" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>AI budget guardrail</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="C53" s="15" t="inlineStr">
         <is>
           <t>Any canvas (AI draft) + the AI usage display</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>Look at the AI-draft buttons and the AI usage display.</t>
         </is>
       </c>
-      <c r="E52" s="15" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
         <is>
           <t>When the workspace is over its daily AI budget, AI-draft buttons show “AI draft paused (until …)” instead of running; the usage display shows tokens used, or “Unlimited” when there’s no cap.</t>
         </is>
       </c>
-      <c r="F52" s="16" t="inlineStr">
+      <c r="F53" s="16" t="inlineStr">
         <is>
           <t>Honest pause — it never pretends to produce an AI result it can’t.</t>
         </is>
       </c>
-      <c r="G52" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H52" s="18" t="inlineStr"/>
-      <c r="I52" s="15" t="inlineStr"/>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="12" t="inlineStr">
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="inlineStr"/>
+      <c r="I53" s="15" t="inlineStr"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="12" t="inlineStr">
         <is>
           <t>6 · Notifications, Journal &amp; Learning</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="92" customHeight="1">
-      <c r="A54" s="13" t="inlineStr">
+    <row r="55" ht="92" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B54" s="14" t="inlineStr">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>Notifications inbox</t>
         </is>
       </c>
-      <c r="C54" s="15" t="inlineStr">
+      <c r="C55" s="15" t="inlineStr">
         <is>
           <t>Bell / Notifications</t>
         </is>
       </c>
-      <c r="D54" s="15" t="inlineStr">
+      <c r="D55" s="15" t="inlineStr">
         <is>
           <t>Open it, mark one read, and “mark all read”.</t>
         </is>
       </c>
-      <c r="E54" s="15" t="inlineStr">
+      <c r="E55" s="15" t="inlineStr">
         <is>
           <t>The unread count updates.</t>
         </is>
       </c>
-      <c r="F54" s="16" t="inlineStr">
+      <c r="F55" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G54" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H54" s="18" t="inlineStr"/>
-      <c r="I54" s="15" t="inlineStr"/>
-    </row>
-    <row r="55" ht="92" customHeight="1">
-      <c r="A55" s="19" t="inlineStr">
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="inlineStr"/>
+      <c r="I55" s="15" t="inlineStr"/>
+    </row>
+    <row r="56" ht="92" customHeight="1">
+      <c r="A56" s="19" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B55" s="20" t="inlineStr">
+      <c r="B56" s="20" t="inlineStr">
         <is>
           <t>Email preferences</t>
         </is>
       </c>
-      <c r="C55" s="21" t="inlineStr">
+      <c r="C56" s="21" t="inlineStr">
         <is>
           <t>Notifications → Preferences</t>
         </is>
       </c>
-      <c r="D55" s="21" t="inlineStr">
+      <c r="D56" s="21" t="inlineStr">
         <is>
           <t>Toggle the master email switch and the 5 category switches.</t>
         </is>
       </c>
-      <c r="E55" s="21" t="inlineStr">
+      <c r="E56" s="21" t="inlineStr">
         <is>
           <t>They save.</t>
         </is>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>The “Digest &amp; quiet hours” and “Announcements” tabs are demo-only for now.</t>
         </is>
       </c>
-      <c r="G55" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H55" s="23" t="inlineStr"/>
-      <c r="I55" s="21" t="inlineStr"/>
-    </row>
-    <row r="56" ht="92" customHeight="1">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="G56" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H56" s="23" t="inlineStr"/>
+      <c r="I56" s="21" t="inlineStr"/>
+    </row>
+    <row r="57" ht="92" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>Read the journal</t>
         </is>
       </c>
-      <c r="C56" s="15" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>Read journal entries.</t>
         </is>
       </c>
-      <c r="E56" s="15" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>Reading works.</t>
         </is>
       </c>
-      <c r="F56" s="16" t="inlineStr">
+      <c r="F57" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G56" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H56" s="18" t="inlineStr"/>
-      <c r="I56" s="15" t="inlineStr"/>
-    </row>
-    <row r="57" ht="92" customHeight="1">
-      <c r="A57" s="19" t="inlineStr">
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H57" s="18" t="inlineStr"/>
+      <c r="I57" s="15" t="inlineStr"/>
+    </row>
+    <row r="58" ht="92" customHeight="1">
+      <c r="A58" s="19" t="inlineStr">
         <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="B57" s="20" t="inlineStr">
+      <c r="B58" s="20" t="inlineStr">
         <is>
           <t>Save a new journal entry</t>
         </is>
       </c>
-      <c r="C57" s="21" t="inlineStr">
+      <c r="C58" s="21" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="D57" s="21" t="inlineStr">
+      <c r="D58" s="21" t="inlineStr">
         <is>
           <t>Try to save a new entry.</t>
         </is>
       </c>
-      <c r="E57" s="21" t="inlineStr">
+      <c r="E58" s="21" t="inlineStr">
         <is>
           <t>It fails gracefully — it doesn’t crash the page.</t>
         </is>
       </c>
-      <c r="F57" s="22" t="inlineStr">
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>Saving isn’t set up on the test server yet — expected to fail softly.</t>
         </is>
       </c>
-      <c r="G57" s="25" t="inlineStr">
+      <c r="G58" s="25" t="inlineStr">
         <is>
           <t>⛔  Not ready (expected)</t>
         </is>
       </c>
-      <c r="H57" s="23" t="inlineStr"/>
-      <c r="I57" s="21" t="inlineStr"/>
-    </row>
-    <row r="58" ht="92" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="H58" s="23" t="inlineStr"/>
+      <c r="I58" s="21" t="inlineStr"/>
+    </row>
+    <row r="59" ht="92" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
         <is>
           <t>6.5</t>
         </is>
       </c>
-      <c r="B58" s="14" t="inlineStr">
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>Learning academy</t>
         </is>
       </c>
-      <c r="C58" s="15" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
         <is>
           <t>Academy</t>
         </is>
       </c>
-      <c r="D58" s="15" t="inlineStr">
+      <c r="D59" s="15" t="inlineStr">
         <is>
           <t>Browse courses / articles / paths / certificates, enroll, and complete a lesson.</t>
         </is>
       </c>
-      <c r="E58" s="15" t="inlineStr">
+      <c r="E59" s="15" t="inlineStr">
         <is>
           <t>These work and save.</t>
         </is>
       </c>
-      <c r="F58" s="16" t="inlineStr">
+      <c r="F59" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G58" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H58" s="18" t="inlineStr"/>
-      <c r="I58" s="15" t="inlineStr"/>
-    </row>
-    <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+      <c r="G59" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H59" s="18" t="inlineStr"/>
+      <c r="I59" s="15" t="inlineStr"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t>7 · Documents</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="92" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
+    <row r="61" ht="92" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>Files</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
+      <c r="C61" s="15" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="D60" s="15" t="inlineStr">
+      <c r="D61" s="15" t="inlineStr">
         <is>
           <t>Upload, list, and delete a file.</t>
         </is>
       </c>
-      <c r="E60" s="15" t="inlineStr">
+      <c r="E61" s="15" t="inlineStr">
         <is>
           <t>All three work.</t>
         </is>
       </c>
-      <c r="F60" s="16" t="inlineStr">
+      <c r="F61" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G60" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H60" s="18" t="inlineStr"/>
-      <c r="I60" s="15" t="inlineStr"/>
-    </row>
-    <row r="61" ht="92" customHeight="1">
-      <c r="A61" s="19" t="inlineStr">
+      <c r="G61" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H61" s="18" t="inlineStr"/>
+      <c r="I61" s="15" t="inlineStr"/>
+    </row>
+    <row r="62" ht="92" customHeight="1">
+      <c r="A62" s="19" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="B61" s="20" t="inlineStr">
+      <c r="B62" s="20" t="inlineStr">
         <is>
           <t>Share a document</t>
         </is>
       </c>
-      <c r="C61" s="21" t="inlineStr">
+      <c r="C62" s="21" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="D61" s="21" t="inlineStr">
+      <c r="D62" s="21" t="inlineStr">
         <is>
           <t>Share a document, then remove the share.</t>
         </is>
       </c>
-      <c r="E61" s="21" t="inlineStr">
+      <c r="E62" s="21" t="inlineStr">
         <is>
           <t>The share list updates.</t>
         </is>
       </c>
-      <c r="F61" s="22" t="inlineStr">
+      <c r="F62" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G61" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H61" s="23" t="inlineStr"/>
-      <c r="I61" s="21" t="inlineStr"/>
-    </row>
-    <row r="62" ht="92" customHeight="1">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="G62" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H62" s="23" t="inlineStr"/>
+      <c r="I62" s="21" t="inlineStr"/>
+    </row>
+    <row r="63" ht="92" customHeight="1">
+      <c r="A63" s="13" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>Signature requests</t>
         </is>
       </c>
-      <c r="C62" s="15" t="inlineStr">
+      <c r="C63" s="15" t="inlineStr">
         <is>
           <t>Documents → Signatures</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
+      <c r="D63" s="15" t="inlineStr">
         <is>
           <t>Send, remind, or cancel a signature request.</t>
         </is>
       </c>
-      <c r="E62" s="15" t="inlineStr">
+      <c r="E63" s="15" t="inlineStr">
         <is>
           <t>The status reflects what you did.</t>
         </is>
       </c>
-      <c r="F62" s="16" t="inlineStr">
+      <c r="F63" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G62" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H62" s="18" t="inlineStr"/>
-      <c r="I62" s="15" t="inlineStr"/>
-    </row>
-    <row r="63" ht="92" customHeight="1">
-      <c r="A63" s="19" t="inlineStr">
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr"/>
+      <c r="I63" s="15" t="inlineStr"/>
+    </row>
+    <row r="64" ht="92" customHeight="1">
+      <c r="A64" s="19" t="inlineStr">
         <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="B63" s="20" t="inlineStr">
+      <c r="B64" s="20" t="inlineStr">
         <is>
           <t>Create from a template</t>
         </is>
       </c>
-      <c r="C63" s="21" t="inlineStr">
+      <c r="C64" s="21" t="inlineStr">
         <is>
           <t>Documents → Templates</t>
         </is>
       </c>
-      <c r="D63" s="21" t="inlineStr">
+      <c r="D64" s="21" t="inlineStr">
         <is>
           <t>Create a document from a template.</t>
         </is>
       </c>
-      <c r="E63" s="21" t="inlineStr">
+      <c r="E64" s="21" t="inlineStr">
         <is>
           <t>It creates the document.</t>
         </is>
       </c>
-      <c r="F63" s="22" t="inlineStr">
+      <c r="F64" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G63" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H63" s="23" t="inlineStr"/>
-      <c r="I63" s="21" t="inlineStr"/>
-    </row>
-    <row r="64" ht="92" customHeight="1">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="G64" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H64" s="23" t="inlineStr"/>
+      <c r="I64" s="21" t="inlineStr"/>
+    </row>
+    <row r="65" ht="92" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
         <is>
           <t>7.5</t>
         </is>
       </c>
-      <c r="B64" s="14" t="inlineStr">
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>Edit &amp; save a document</t>
         </is>
       </c>
-      <c r="C64" s="15" t="inlineStr">
+      <c r="C65" s="15" t="inlineStr">
         <is>
           <t>Documents → open a document</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
+      <c r="D65" s="15" t="inlineStr">
         <is>
           <t>Open the editor, make edits, and save.</t>
         </is>
       </c>
-      <c r="E64" s="15" t="inlineStr">
+      <c r="E65" s="15" t="inlineStr">
         <is>
           <t>Your edits save.</t>
         </is>
       </c>
-      <c r="F64" s="16" t="inlineStr">
+      <c r="F65" s="16" t="inlineStr">
         <is>
           <t>Documents don’t auto-save — click Save. If it was changed elsewhere you get a “reload” banner and it won’t overwrite.</t>
         </is>
       </c>
-      <c r="G64" s="24" t="inlineStr">
+      <c r="G65" s="24" t="inlineStr">
         <is>
           <t>⚠️  Works, watch out</t>
         </is>
       </c>
-      <c r="H64" s="18" t="inlineStr"/>
-      <c r="I64" s="15" t="inlineStr"/>
-    </row>
-    <row r="65" ht="92" customHeight="1">
-      <c r="A65" s="19" t="inlineStr">
+      <c r="H65" s="18" t="inlineStr"/>
+      <c r="I65" s="15" t="inlineStr"/>
+    </row>
+    <row r="66" ht="92" customHeight="1">
+      <c r="A66" s="19" t="inlineStr">
         <is>
           <t>7.6</t>
         </is>
       </c>
-      <c r="B65" s="20" t="inlineStr">
+      <c r="B66" s="20" t="inlineStr">
         <is>
           <t>Open a real emailed sign/share link</t>
         </is>
       </c>
-      <c r="C65" s="21" t="inlineStr">
+      <c r="C66" s="21" t="inlineStr">
         <is>
           <t>The sign/share link</t>
         </is>
       </c>
-      <c r="D65" s="21" t="inlineStr">
+      <c r="D66" s="21" t="inlineStr">
         <is>
           <t>Open a real emailed link.</t>
         </is>
       </c>
-      <c r="E65" s="21" t="inlineStr">
+      <c r="E66" s="21" t="inlineStr">
         <is>
           <t>The recipient page works when opened on the app website.</t>
         </is>
       </c>
-      <c r="F65" s="22" t="inlineStr">
+      <c r="F66" s="22" t="inlineStr">
         <is>
           <t>Straight from an email it may show a raw data page — open it on the app website instead.</t>
         </is>
       </c>
-      <c r="G65" s="25" t="inlineStr">
+      <c r="G66" s="25" t="inlineStr">
         <is>
           <t>⛔  Not ready (expected)</t>
         </is>
       </c>
-      <c r="H65" s="23" t="inlineStr"/>
-      <c r="I65" s="21" t="inlineStr"/>
-    </row>
-    <row r="66" ht="92" customHeight="1">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="H66" s="23" t="inlineStr"/>
+      <c r="I66" s="21" t="inlineStr"/>
+    </row>
+    <row r="67" ht="92" customHeight="1">
+      <c r="A67" s="13" t="inlineStr">
         <is>
           <t>7.7</t>
         </is>
       </c>
-      <c r="B66" s="14" t="inlineStr">
+      <c r="B67" s="14" t="inlineStr">
         <is>
           <t>Edit a document’s sections</t>
         </is>
       </c>
-      <c r="C66" s="15" t="inlineStr">
+      <c r="C67" s="15" t="inlineStr">
         <is>
           <t>Documents → open a document</t>
         </is>
       </c>
-      <c r="D66" s="15" t="inlineStr">
+      <c r="D67" s="15" t="inlineStr">
         <is>
           <t>Add a section, delete one, drag a section to reorder (or use the up/down arrows), and rename a heading. Then Save.</t>
         </is>
       </c>
-      <c r="E66" s="15" t="inlineStr">
+      <c r="E67" s="15" t="inlineStr">
         <is>
           <t>All the section changes save after you click Save.</t>
         </is>
       </c>
-      <c r="F66" s="16" t="inlineStr">
+      <c r="F67" s="16" t="inlineStr">
         <is>
           <t>Documents don’t auto-save — you must click Save. Headings used to be read-only.</t>
         </is>
       </c>
-      <c r="G66" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H66" s="18" t="inlineStr"/>
-      <c r="I66" s="15" t="inlineStr"/>
-    </row>
-    <row r="67" ht="92" customHeight="1">
-      <c r="A67" s="19" t="inlineStr">
+      <c r="G67" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H67" s="18" t="inlineStr"/>
+      <c r="I67" s="15" t="inlineStr"/>
+    </row>
+    <row r="68" ht="92" customHeight="1">
+      <c r="A68" s="19" t="inlineStr">
         <is>
           <t>7.8</t>
         </is>
       </c>
-      <c r="B67" s="20" t="inlineStr">
+      <c r="B68" s="20" t="inlineStr">
         <is>
           <t>Sign a document</t>
         </is>
       </c>
-      <c r="C67" s="21" t="inlineStr">
+      <c r="C68" s="21" t="inlineStr">
         <is>
           <t>The signing link, on the app website</t>
         </is>
       </c>
-      <c r="D67" s="21" t="inlineStr">
+      <c r="D68" s="21" t="inlineStr">
         <is>
           <t>Read the preview, type your full name (shown styled like a signature), tick the “I agree…” box, then Sign.</t>
         </is>
       </c>
-      <c r="E67" s="21" t="inlineStr">
+      <c r="E68" s="21" t="inlineStr">
         <is>
           <t>Your typed name is accepted and you see a “signed — thank you” confirmation.</t>
         </is>
       </c>
-      <c r="F67" s="22" t="inlineStr">
+      <c r="F68" s="22" t="inlineStr">
         <is>
           <t>It’s a typed signature (no drawing pad). The Sign button stays disabled until you tick consent.</t>
         </is>
       </c>
-      <c r="G67" s="17" t="inlineStr">
-        <is>
-          <t>✅  Works</t>
-        </is>
-      </c>
-      <c r="H67" s="23" t="inlineStr"/>
-      <c r="I67" s="21" t="inlineStr"/>
+      <c r="G68" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
+        </is>
+      </c>
+      <c r="H68" s="23" t="inlineStr"/>
+      <c r="I68" s="21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="A59:I59"/>
-    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A60:I60"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A23:I23"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A53:I53"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
+    <dataValidation sqref="H4:H68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3287,7 +3326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3388,10 +3427,22 @@
     <row r="10" ht="50" customHeight="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
+          <t>AI Co-Founder chat</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>The chat on the AI Co-Founder page (and the floating button) says “coming soon” and can’t answer yet — the chat has no backend. The real AI still powers your dashboard briefing, mission reasons and health tips (test 1.19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
           <t>Demo-only areas (placeholder data)</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>Not connected to real data yet — don’t test as real: Marketing, Sales, Finance, Validation, Funding, Investor Readiness, Legal &amp; Compliance, Calendar, Analytics &amp; Reports, Marketplace, Admin / Super-Admin, and the Notifications “Digest / quiet hours” &amp; “Announcements” tabs.</t>
         </is>

</xml_diff>

<commit_message>
Wire Validation Hub slice 2: Interviews (real API)
- lib/api/validation.ts: listInterviews / createInterview / updateInterview
  + RawInterview/CreateInterviewBody (GET/POST/PATCH /validation/interviews)
- hooks/useInterviews.ts (new): load on mount, addInterview (POST -> prepend),
  maps key_quotes[0] -> quote; honest error state
- interviews/page.tsx: rewired to the real hook; the New-note form POSTs
  (held_on=today, verdict=lowercased stance, key_quotes=[quote] since the API
  422s on empty quotes); list reads real data with honest empty/loading/error

Verified live: added 'Ada / fintech / Supports / I would pay for this today'
(POST 201), persisted on reload. The Synthesize insights button stays mock
(AI synthesize is slice 5).

Docs: SOP module-41 (slice 2), frontend checklist, QA checklist 8.2 + xlsx.
</commit_message>
<xml_diff>
--- a/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
+++ b/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
@@ -882,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3393,36 +3393,75 @@
       </c>
       <c r="B72" s="20" t="inlineStr">
         <is>
-          <t>Rest of Validation Hub</t>
+          <t>Interview notes</t>
         </is>
       </c>
       <c r="C72" s="21" t="inlineStr">
         <is>
-          <t>Validation Hub → Interviews / Surveys / Smoke tests / Interview scripts</t>
+          <t>Validation Hub → Interviews</t>
         </is>
       </c>
       <c r="D72" s="21" t="inlineStr">
         <is>
-          <t>(Nothing to test yet.)</t>
+          <t>Fill in the New-note form (who you spoke to, a segment tag, a key quote, and pick Supports / Contradicts / Neutral), then Save note.</t>
         </is>
       </c>
       <c r="E72" s="21" t="inlineStr">
         <is>
-          <t>These are still being connected.</t>
+          <t>Your note is saved and appears on the right with the name, segment, a coloured stance badge and the quote. It’s still there after a reload.</t>
         </is>
       </c>
       <c r="F72" s="22" t="inlineStr">
         <is>
-          <t>Interviews, Surveys, Smoke tests and Interview scripts are being wired next — treat as not-ready for now.</t>
-        </is>
-      </c>
-      <c r="G72" s="25" t="inlineStr">
-        <is>
-          <t>⛔  Not ready (expected)</t>
+          <t>A quote is required (an empty one is rejected). The empty list shows a friendly prompt. The “Synthesize insights” button isn’t connected yet.</t>
+        </is>
+      </c>
+      <c r="G72" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
         </is>
       </c>
       <c r="H72" s="23" t="inlineStr"/>
       <c r="I72" s="21" t="inlineStr"/>
+    </row>
+    <row r="73" ht="92" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>Rest of Validation Hub</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>Validation Hub → Surveys / Smoke tests / Interview scripts</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>(Nothing to test yet.)</t>
+        </is>
+      </c>
+      <c r="E73" s="15" t="inlineStr">
+        <is>
+          <t>These are still being connected.</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>Surveys, Smoke tests and Interview scripts are being wired next — treat as not-ready for now.</t>
+        </is>
+      </c>
+      <c r="G73" s="25" t="inlineStr">
+        <is>
+          <t>⛔  Not ready (expected)</t>
+        </is>
+      </c>
+      <c r="H73" s="18" t="inlineStr"/>
+      <c r="I73" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3437,7 +3476,7 @@
     <mergeCell ref="A30:I30"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
+    <dataValidation sqref="H4:H73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Wire Validation Hub slice 3b: public survey response page
Completes the surveys loop (guide §5). New no-auth page app/s/[token]:

- GET /validation/surveys/{token} renders a branded, chrome-less form:
  choice (radios), scale (1-5), nps (0-10), open (textarea, 4000 cap)
- POST /validation/surveys/{token}/responses with {answers:{qid:value}}
- States: loading; uniform 404 'not available' (unknown/draft/closed are
  indistinguishable by design); 429 'too many submissions'; 422 surfaces
  the first field_error; 'Thank you' success. Client-side required check.

Verified live end-to-end: created+opened a survey -> visited /s/{token} ->
answered (choice Yes, NPS 9) -> Thank you -> owner analytics showed
responses:1, completion 100%, {Yes:1,No:0}, NPS avg 9.0.

Surveys slice (3a owner + 3b public) is now a complete create->share->
respond->analytics loop.

Docs: SOP module-41 (slice 3b), frontend checklist, QA checklist 8.4 + xlsx.
</commit_message>
<xml_diff>
--- a/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
+++ b/docs/checklist/Cofoundaz_QA_Test_Sheet.xlsx
@@ -882,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3471,36 +3471,75 @@
       </c>
       <c r="B74" s="20" t="inlineStr">
         <is>
-          <t>Rest of Validation Hub</t>
+          <t>Answer a survey (public link)</t>
         </is>
       </c>
       <c r="C74" s="21" t="inlineStr">
         <is>
-          <t>Validation Hub → the public survey link / Smoke tests / Interview scripts</t>
+          <t>The survey share link from test 8.3</t>
         </is>
       </c>
       <c r="D74" s="21" t="inlineStr">
         <is>
-          <t>(Nothing to test yet.)</t>
+          <t>Open the share link in any browser (you can even be logged out). Answer the questions and press Submit.</t>
         </is>
       </c>
       <c r="E74" s="21" t="inlineStr">
         <is>
-          <t>These are still being connected.</t>
+          <t>You see the questions, can answer them, and get a “Thank you”. Back in the app, that survey’s results (test 8.3) now count your answer.</t>
         </is>
       </c>
       <c r="F74" s="22" t="inlineStr">
         <is>
-          <t>The public survey-answer page, Smoke tests and Interview scripts are being wired next — treat as not-ready for now.</t>
-        </is>
-      </c>
-      <c r="G74" s="25" t="inlineStr">
-        <is>
-          <t>⛔  Not ready (expected)</t>
+          <t>No login needed. A wrong or closed link just says “not available”. Required questions must be answered before you can submit.</t>
+        </is>
+      </c>
+      <c r="G74" s="17" t="inlineStr">
+        <is>
+          <t>✅  Works</t>
         </is>
       </c>
       <c r="H74" s="23" t="inlineStr"/>
       <c r="I74" s="21" t="inlineStr"/>
+    </row>
+    <row r="75" ht="92" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>Rest of Validation Hub</t>
+        </is>
+      </c>
+      <c r="C75" s="15" t="inlineStr">
+        <is>
+          <t>Validation Hub → Smoke tests / Interview scripts</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>(Nothing to test yet.)</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>These are still being connected.</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>Smoke tests and Interview scripts are being wired next — treat as not-ready for now.</t>
+        </is>
+      </c>
+      <c r="G75" s="25" t="inlineStr">
+        <is>
+          <t>⛔  Not ready (expected)</t>
+        </is>
+      </c>
+      <c r="H75" s="18" t="inlineStr"/>
+      <c r="I75" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3515,7 +3554,7 @@
     <mergeCell ref="A30:I30"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
+    <dataValidation sqref="H4:H75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Result" prompt="Pick one" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>